<commit_message>
Add Mary Alice Thoren ancestry
</commit_message>
<xml_diff>
--- a/original-data/final-family-tree/Fredric_Vollmer_Complete_Family_Tree_Index.xlsx
+++ b/original-data/final-family-tree/Fredric_Vollmer_Complete_Family_Tree_Index.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R313a684ad754461d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancestor Index" sheetId="2" r:id="R2eb0ab1114804406"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="3" r:id="R5173f70a21e14852"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended Family" sheetId="4" r:id="R28d380c825bd4366"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household Audit" sheetId="5" r:id="R0ad3fe7585344163"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correction Log" sheetId="6" r:id="R2f9211f8ce7a4ca0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Gaps" sheetId="7" r:id="R348649b970b547a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Key" sheetId="8" r:id="R0ec899dba3ba421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated People" sheetId="9" r:id="R38bc328353c741b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Families" sheetId="10" r:id="R823654161d254f64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Sources" sheetId="11" r:id="Rf58ac1acd71c4bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Overview" sheetId="12" r:id="Rf07c277ad4b146bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rd876436d6c344821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancestor Index" sheetId="2" r:id="Raedecbfabe5244df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="3" r:id="R9724e9810991473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended Family" sheetId="4" r:id="Rbd782cfff06848ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household Audit" sheetId="5" r:id="R35014b64b8884ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correction Log" sheetId="6" r:id="R079ee3222f5b48c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Gaps" sheetId="7" r:id="Re8853001e90f4d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Key" sheetId="8" r:id="R0aad920191204719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated People" sheetId="9" r:id="Rbdf6ed21aad04bdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Families" sheetId="10" r:id="Ra891baee4ff74c84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Sources" sheetId="11" r:id="Rc62711123b0943d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Overview" sheetId="12" r:id="R73a3aaa9ebd34d98"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -678,7 +678,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c26b32e712e4f68"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5fd8d5d2a1e94dae"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -714,8 +714,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ConsolidatedSourcesTable" displayName="ConsolidatedSourcesTable" ref="A1:F73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F73"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ConsolidatedSourcesTable" displayName="ConsolidatedSourcesTable" ref="A1:F77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F77"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="source_id"/>
     <x:tableColumn id="2" name="title"/>
@@ -825,8 +825,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ConsolidatedPeopleTable" displayName="ConsolidatedPeopleTable" ref="A1:J309" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J309"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ConsolidatedPeopleTable" displayName="ConsolidatedPeopleTable" ref="A1:J311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J311"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="individual_id"/>
     <x:tableColumn id="2" name="name"/>
@@ -844,15 +844,16 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ConsolidatedFamiliesTable" displayName="ConsolidatedFamiliesTable" ref="A1:F145" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F145"/>
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ConsolidatedFamiliesTable" displayName="ConsolidatedFamiliesTable" ref="A1:G147" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G147"/>
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="family_id"/>
     <x:tableColumn id="2" name="husband_id"/>
     <x:tableColumn id="3" name="wife_id"/>
     <x:tableColumn id="4" name="children_ids"/>
-    <x:tableColumn id="5" name="notes"/>
-    <x:tableColumn id="6" name="source_refs"/>
+    <x:tableColumn id="5" name="marriage"/>
+    <x:tableColumn id="6" name="notes"/>
+    <x:tableColumn id="7" name="source_refs"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1533,7 +1534,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R665b9ecbf1a84250"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R802a8f5369b74a0e"/>
 </x:worksheet>
 </file>
 
@@ -1545,8 +1546,9 @@
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="72" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="72" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1563,9 +1565,12 @@
         <x:v>children_ids</x:v>
       </x:c>
       <x:c r="E1" s="102" t="str">
+        <x:v>marriage</x:v>
+      </x:c>
+      <x:c r="F1" s="102" t="str">
         <x:v>notes</x:v>
       </x:c>
-      <x:c r="F1" s="102" t="str">
+      <x:c r="G1" s="102" t="str">
         <x:v>source_refs</x:v>
       </x:c>
     </x:row>
@@ -1582,10 +1587,11 @@
       <x:c r="D2" s="97" t="str">
         <x:v>I002;I177</x:v>
       </x:c>
-      <x:c r="E2" s="97" t="str">
+      <x:c r="E2" s="97" t="str"/>
+      <x:c r="F2" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F2" s="97" t="str">
+      <x:c r="G2" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -1602,10 +1608,11 @@
       <x:c r="D3" s="97" t="str">
         <x:v>I003;I178;I183</x:v>
       </x:c>
-      <x:c r="E3" s="97" t="str">
+      <x:c r="E3" s="97" t="str"/>
+      <x:c r="F3" s="97" t="str">
         <x:v>Children reconstructed from the 1998 Art Muller family chart. | Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F3" s="97" t="str">
+      <x:c r="G3" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -1622,10 +1629,11 @@
       <x:c r="D4" s="97" t="str">
         <x:v>I004;I193;I200;I202</x:v>
       </x:c>
-      <x:c r="E4" s="97" t="str">
+      <x:c r="E4" s="97" t="str"/>
+      <x:c r="F4" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package. | Four-child McCormick sibling set; Gwen is a core sibling.</x:v>
       </x:c>
-      <x:c r="F4" s="97" t="str">
+      <x:c r="G4" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -1642,10 +1650,11 @@
       <x:c r="D5" s="97" t="str">
         <x:v>I005;I310;I311</x:v>
       </x:c>
-      <x:c r="E5" s="97" t="str">
+      <x:c r="E5" s="97" t="str"/>
+      <x:c r="F5" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F5" s="97" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -1662,10 +1671,11 @@
       <x:c r="D6" s="97" t="str">
         <x:v>I006;I314;I315</x:v>
       </x:c>
-      <x:c r="E6" s="97" t="str">
+      <x:c r="E6" s="97" t="str"/>
+      <x:c r="F6" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F6" s="97" t="str">
+      <x:c r="G6" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -1684,6 +1694,7 @@
       </x:c>
       <x:c r="E7" s="97" t="str"/>
       <x:c r="F7" s="97" t="str"/>
+      <x:c r="G7" s="97" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="97" t="str">
@@ -1700,6 +1711,7 @@
       </x:c>
       <x:c r="E8" s="97" t="str"/>
       <x:c r="F8" s="97" t="str"/>
+      <x:c r="G8" s="97" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="97" t="str">
@@ -1714,6 +1726,7 @@
       </x:c>
       <x:c r="E9" s="97" t="str"/>
       <x:c r="F9" s="97" t="str"/>
+      <x:c r="G9" s="97" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="97" t="str">
@@ -1730,6 +1743,7 @@
       </x:c>
       <x:c r="E10" s="97" t="str"/>
       <x:c r="F10" s="97" t="str"/>
+      <x:c r="G10" s="97" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="97" t="str">
@@ -1746,6 +1760,7 @@
       </x:c>
       <x:c r="E11" s="97" t="str"/>
       <x:c r="F11" s="97" t="str"/>
+      <x:c r="G11" s="97" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="97" t="str">
@@ -1762,6 +1777,7 @@
       </x:c>
       <x:c r="E12" s="97" t="str"/>
       <x:c r="F12" s="97" t="str"/>
+      <x:c r="G12" s="97" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="97" t="str">
@@ -1778,6 +1794,7 @@
       </x:c>
       <x:c r="E13" s="97" t="str"/>
       <x:c r="F13" s="97" t="str"/>
+      <x:c r="G13" s="97" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="97" t="str">
@@ -1794,6 +1811,7 @@
       </x:c>
       <x:c r="E14" s="97" t="str"/>
       <x:c r="F14" s="97" t="str"/>
+      <x:c r="G14" s="97" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="97" t="str">
@@ -1810,6 +1828,7 @@
       </x:c>
       <x:c r="E15" s="97" t="str"/>
       <x:c r="F15" s="97" t="str"/>
+      <x:c r="G15" s="97" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="97" t="str">
@@ -1826,6 +1845,7 @@
       </x:c>
       <x:c r="E16" s="97" t="str"/>
       <x:c r="F16" s="97" t="str"/>
+      <x:c r="G16" s="97" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="97" t="str">
@@ -1842,6 +1862,7 @@
       </x:c>
       <x:c r="E17" s="97" t="str"/>
       <x:c r="F17" s="97" t="str"/>
+      <x:c r="G17" s="97" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="97" t="str">
@@ -1856,6 +1877,7 @@
       </x:c>
       <x:c r="E18" s="97" t="str"/>
       <x:c r="F18" s="97" t="str"/>
+      <x:c r="G18" s="97" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="97" t="str">
@@ -1872,6 +1894,7 @@
       </x:c>
       <x:c r="E19" s="97" t="str"/>
       <x:c r="F19" s="97" t="str"/>
+      <x:c r="G19" s="97" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="97" t="str">
@@ -1888,6 +1911,7 @@
       </x:c>
       <x:c r="E20" s="97" t="str"/>
       <x:c r="F20" s="97" t="str"/>
+      <x:c r="G20" s="97" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="97" t="str">
@@ -1904,6 +1928,7 @@
       </x:c>
       <x:c r="E21" s="97" t="str"/>
       <x:c r="F21" s="97" t="str"/>
+      <x:c r="G21" s="97" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="97" t="str">
@@ -1918,6 +1943,7 @@
       </x:c>
       <x:c r="E22" s="97" t="str"/>
       <x:c r="F22" s="97" t="str"/>
+      <x:c r="G22" s="97" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="97" t="str">
@@ -1934,6 +1960,7 @@
       </x:c>
       <x:c r="E23" s="97" t="str"/>
       <x:c r="F23" s="97" t="str"/>
+      <x:c r="G23" s="97" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="97" t="str">
@@ -1950,6 +1977,7 @@
       </x:c>
       <x:c r="E24" s="97" t="str"/>
       <x:c r="F24" s="97" t="str"/>
+      <x:c r="G24" s="97" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="97" t="str">
@@ -1966,6 +1994,7 @@
       </x:c>
       <x:c r="E25" s="97" t="str"/>
       <x:c r="F25" s="97" t="str"/>
+      <x:c r="G25" s="97" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="97" t="str">
@@ -1980,6 +2009,7 @@
       </x:c>
       <x:c r="E26" s="97" t="str"/>
       <x:c r="F26" s="97" t="str"/>
+      <x:c r="G26" s="97" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="97" t="str">
@@ -1996,6 +2026,7 @@
       </x:c>
       <x:c r="E27" s="97" t="str"/>
       <x:c r="F27" s="97" t="str"/>
+      <x:c r="G27" s="97" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="97" t="str">
@@ -2012,6 +2043,7 @@
       </x:c>
       <x:c r="E28" s="97" t="str"/>
       <x:c r="F28" s="97" t="str"/>
+      <x:c r="G28" s="97" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="97" t="str">
@@ -2028,6 +2060,7 @@
       </x:c>
       <x:c r="E29" s="97" t="str"/>
       <x:c r="F29" s="97" t="str"/>
+      <x:c r="G29" s="97" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="97" t="str">
@@ -2044,6 +2077,7 @@
       </x:c>
       <x:c r="E30" s="97" t="str"/>
       <x:c r="F30" s="97" t="str"/>
+      <x:c r="G30" s="97" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="97" t="str">
@@ -2060,6 +2094,7 @@
       </x:c>
       <x:c r="E31" s="97" t="str"/>
       <x:c r="F31" s="97" t="str"/>
+      <x:c r="G31" s="97" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="97" t="str">
@@ -2076,6 +2111,7 @@
       </x:c>
       <x:c r="E32" s="97" t="str"/>
       <x:c r="F32" s="97" t="str"/>
+      <x:c r="G32" s="97" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="97" t="str">
@@ -2092,6 +2128,7 @@
       </x:c>
       <x:c r="E33" s="97" t="str"/>
       <x:c r="F33" s="97" t="str"/>
+      <x:c r="G33" s="97" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="97" t="str">
@@ -2108,6 +2145,7 @@
       </x:c>
       <x:c r="E34" s="97" t="str"/>
       <x:c r="F34" s="97" t="str"/>
+      <x:c r="G34" s="97" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="97" t="str">
@@ -2124,6 +2162,7 @@
       </x:c>
       <x:c r="E35" s="97" t="str"/>
       <x:c r="F35" s="97" t="str"/>
+      <x:c r="G35" s="97" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="97" t="str">
@@ -2140,6 +2179,7 @@
       </x:c>
       <x:c r="E36" s="97" t="str"/>
       <x:c r="F36" s="97" t="str"/>
+      <x:c r="G36" s="97" t="str"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="97" t="str">
@@ -2156,6 +2196,7 @@
       </x:c>
       <x:c r="E37" s="97" t="str"/>
       <x:c r="F37" s="97" t="str"/>
+      <x:c r="G37" s="97" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="97" t="str">
@@ -2172,6 +2213,7 @@
       </x:c>
       <x:c r="E38" s="97" t="str"/>
       <x:c r="F38" s="97" t="str"/>
+      <x:c r="G38" s="97" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="97" t="str">
@@ -2188,6 +2230,7 @@
       </x:c>
       <x:c r="E39" s="97" t="str"/>
       <x:c r="F39" s="97" t="str"/>
+      <x:c r="G39" s="97" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="97" t="str">
@@ -2204,6 +2247,7 @@
       </x:c>
       <x:c r="E40" s="97" t="str"/>
       <x:c r="F40" s="97" t="str"/>
+      <x:c r="G40" s="97" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="97" t="str">
@@ -2220,6 +2264,7 @@
       </x:c>
       <x:c r="E41" s="97" t="str"/>
       <x:c r="F41" s="97" t="str"/>
+      <x:c r="G41" s="97" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="97" t="str">
@@ -2234,6 +2279,7 @@
       </x:c>
       <x:c r="E42" s="97" t="str"/>
       <x:c r="F42" s="97" t="str"/>
+      <x:c r="G42" s="97" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="97" t="str">
@@ -2250,6 +2296,7 @@
       </x:c>
       <x:c r="E43" s="97" t="str"/>
       <x:c r="F43" s="97" t="str"/>
+      <x:c r="G43" s="97" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="97" t="str">
@@ -2266,6 +2313,7 @@
       </x:c>
       <x:c r="E44" s="97" t="str"/>
       <x:c r="F44" s="97" t="str"/>
+      <x:c r="G44" s="97" t="str"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="97" t="str">
@@ -2282,6 +2330,7 @@
       </x:c>
       <x:c r="E45" s="97" t="str"/>
       <x:c r="F45" s="97" t="str"/>
+      <x:c r="G45" s="97" t="str"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="97" t="str">
@@ -2296,6 +2345,7 @@
       </x:c>
       <x:c r="E46" s="97" t="str"/>
       <x:c r="F46" s="97" t="str"/>
+      <x:c r="G46" s="97" t="str"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="97" t="str">
@@ -2312,6 +2362,7 @@
       </x:c>
       <x:c r="E47" s="97" t="str"/>
       <x:c r="F47" s="97" t="str"/>
+      <x:c r="G47" s="97" t="str"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="97" t="str">
@@ -2326,6 +2377,7 @@
       </x:c>
       <x:c r="E48" s="97" t="str"/>
       <x:c r="F48" s="97" t="str"/>
+      <x:c r="G48" s="97" t="str"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="97" t="str">
@@ -2342,6 +2394,7 @@
       </x:c>
       <x:c r="E49" s="97" t="str"/>
       <x:c r="F49" s="97" t="str"/>
+      <x:c r="G49" s="97" t="str"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="97" t="str">
@@ -2358,6 +2411,7 @@
       </x:c>
       <x:c r="E50" s="97" t="str"/>
       <x:c r="F50" s="97" t="str"/>
+      <x:c r="G50" s="97" t="str"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="97" t="str">
@@ -2372,6 +2426,7 @@
       </x:c>
       <x:c r="E51" s="97" t="str"/>
       <x:c r="F51" s="97" t="str"/>
+      <x:c r="G51" s="97" t="str"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="97" t="str">
@@ -2388,6 +2443,7 @@
       </x:c>
       <x:c r="E52" s="97" t="str"/>
       <x:c r="F52" s="97" t="str"/>
+      <x:c r="G52" s="97" t="str"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="97" t="str">
@@ -2404,6 +2460,7 @@
       </x:c>
       <x:c r="E53" s="97" t="str"/>
       <x:c r="F53" s="97" t="str"/>
+      <x:c r="G53" s="97" t="str"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="97" t="str">
@@ -2420,6 +2477,7 @@
       </x:c>
       <x:c r="E54" s="97" t="str"/>
       <x:c r="F54" s="97" t="str"/>
+      <x:c r="G54" s="97" t="str"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="97" t="str">
@@ -2436,6 +2494,7 @@
       </x:c>
       <x:c r="E55" s="97" t="str"/>
       <x:c r="F55" s="97" t="str"/>
+      <x:c r="G55" s="97" t="str"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="97" t="str">
@@ -2452,6 +2511,7 @@
       </x:c>
       <x:c r="E56" s="97" t="str"/>
       <x:c r="F56" s="97" t="str"/>
+      <x:c r="G56" s="97" t="str"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="97" t="str">
@@ -2466,6 +2526,7 @@
       </x:c>
       <x:c r="E57" s="97" t="str"/>
       <x:c r="F57" s="97" t="str"/>
+      <x:c r="G57" s="97" t="str"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="97" t="str">
@@ -2482,6 +2543,7 @@
       </x:c>
       <x:c r="E58" s="97" t="str"/>
       <x:c r="F58" s="97" t="str"/>
+      <x:c r="G58" s="97" t="str"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="97" t="str">
@@ -2498,6 +2560,7 @@
       </x:c>
       <x:c r="E59" s="97" t="str"/>
       <x:c r="F59" s="97" t="str"/>
+      <x:c r="G59" s="97" t="str"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="97" t="str">
@@ -2514,6 +2577,7 @@
       </x:c>
       <x:c r="E60" s="97" t="str"/>
       <x:c r="F60" s="97" t="str"/>
+      <x:c r="G60" s="97" t="str"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="97" t="str">
@@ -2528,10 +2592,11 @@
       <x:c r="D61" s="97" t="str">
         <x:v>I007;I320;I324</x:v>
       </x:c>
-      <x:c r="E61" s="97" t="str">
+      <x:c r="E61" s="97" t="str"/>
+      <x:c r="F61" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F61" s="97" t="str">
+      <x:c r="G61" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -2550,6 +2615,7 @@
       </x:c>
       <x:c r="E62" s="97" t="str"/>
       <x:c r="F62" s="97" t="str"/>
+      <x:c r="G62" s="97" t="str"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="97" t="str">
@@ -2566,6 +2632,7 @@
       </x:c>
       <x:c r="E63" s="97" t="str"/>
       <x:c r="F63" s="97" t="str"/>
+      <x:c r="G63" s="97" t="str"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="97" t="str">
@@ -2582,6 +2649,7 @@
       </x:c>
       <x:c r="E64" s="97" t="str"/>
       <x:c r="F64" s="97" t="str"/>
+      <x:c r="G64" s="97" t="str"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="97" t="str">
@@ -2598,6 +2666,7 @@
       </x:c>
       <x:c r="E65" s="97" t="str"/>
       <x:c r="F65" s="97" t="str"/>
+      <x:c r="G65" s="97" t="str"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="97" t="str">
@@ -2614,6 +2683,7 @@
       </x:c>
       <x:c r="E66" s="97" t="str"/>
       <x:c r="F66" s="97" t="str"/>
+      <x:c r="G66" s="97" t="str"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="97" t="str">
@@ -2628,6 +2698,7 @@
       </x:c>
       <x:c r="E67" s="97" t="str"/>
       <x:c r="F67" s="97" t="str"/>
+      <x:c r="G67" s="97" t="str"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="97" t="str">
@@ -2644,6 +2715,7 @@
       </x:c>
       <x:c r="E68" s="97" t="str"/>
       <x:c r="F68" s="97" t="str"/>
+      <x:c r="G68" s="97" t="str"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="97" t="str">
@@ -2660,6 +2732,7 @@
       </x:c>
       <x:c r="E69" s="97" t="str"/>
       <x:c r="F69" s="97" t="str"/>
+      <x:c r="G69" s="97" t="str"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="97" t="str">
@@ -2674,10 +2747,11 @@
       <x:c r="D70" s="97" t="str">
         <x:v>I008;I327;I328;I329;I332;I333</x:v>
       </x:c>
-      <x:c r="E70" s="97" t="str">
+      <x:c r="E70" s="97" t="str"/>
+      <x:c r="F70" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F70" s="97" t="str">
+      <x:c r="G70" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -2696,6 +2770,7 @@
       </x:c>
       <x:c r="E71" s="97" t="str"/>
       <x:c r="F71" s="97" t="str"/>
+      <x:c r="G71" s="97" t="str"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="97" t="str">
@@ -2712,6 +2787,7 @@
       </x:c>
       <x:c r="E72" s="97" t="str"/>
       <x:c r="F72" s="97" t="str"/>
+      <x:c r="G72" s="97" t="str"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="97" t="str">
@@ -2728,6 +2804,7 @@
       </x:c>
       <x:c r="E73" s="97" t="str"/>
       <x:c r="F73" s="97" t="str"/>
+      <x:c r="G73" s="97" t="str"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="97" t="str">
@@ -2744,6 +2821,7 @@
       </x:c>
       <x:c r="E74" s="97" t="str"/>
       <x:c r="F74" s="97" t="str"/>
+      <x:c r="G74" s="97" t="str"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="97" t="str">
@@ -2760,6 +2838,7 @@
       </x:c>
       <x:c r="E75" s="97" t="str"/>
       <x:c r="F75" s="97" t="str"/>
+      <x:c r="G75" s="97" t="str"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="97" t="str">
@@ -2776,6 +2855,7 @@
       </x:c>
       <x:c r="E76" s="97" t="str"/>
       <x:c r="F76" s="97" t="str"/>
+      <x:c r="G76" s="97" t="str"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="97" t="str">
@@ -2792,6 +2872,7 @@
       </x:c>
       <x:c r="E77" s="97" t="str"/>
       <x:c r="F77" s="97" t="str"/>
+      <x:c r="G77" s="97" t="str"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="97" t="str">
@@ -2808,6 +2889,7 @@
       </x:c>
       <x:c r="E78" s="97" t="str"/>
       <x:c r="F78" s="97" t="str"/>
+      <x:c r="G78" s="97" t="str"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="97" t="str">
@@ -2824,6 +2906,7 @@
       </x:c>
       <x:c r="E79" s="97" t="str"/>
       <x:c r="F79" s="97" t="str"/>
+      <x:c r="G79" s="97" t="str"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="97" t="str">
@@ -2838,6 +2921,7 @@
       </x:c>
       <x:c r="E80" s="97" t="str"/>
       <x:c r="F80" s="97" t="str"/>
+      <x:c r="G80" s="97" t="str"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="97" t="str">
@@ -2854,6 +2938,7 @@
       </x:c>
       <x:c r="E81" s="97" t="str"/>
       <x:c r="F81" s="97" t="str"/>
+      <x:c r="G81" s="97" t="str"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="97" t="str">
@@ -2870,6 +2955,7 @@
       </x:c>
       <x:c r="E82" s="97" t="str"/>
       <x:c r="F82" s="97" t="str"/>
+      <x:c r="G82" s="97" t="str"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="97" t="str">
@@ -2884,6 +2970,7 @@
       </x:c>
       <x:c r="E83" s="97" t="str"/>
       <x:c r="F83" s="97" t="str"/>
+      <x:c r="G83" s="97" t="str"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="97" t="str">
@@ -2900,6 +2987,7 @@
       </x:c>
       <x:c r="E84" s="97" t="str"/>
       <x:c r="F84" s="97" t="str"/>
+      <x:c r="G84" s="97" t="str"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="97" t="str">
@@ -2914,6 +3002,7 @@
       </x:c>
       <x:c r="E85" s="97" t="str"/>
       <x:c r="F85" s="97" t="str"/>
+      <x:c r="G85" s="97" t="str"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="97" t="str">
@@ -2930,6 +3019,7 @@
       </x:c>
       <x:c r="E86" s="97" t="str"/>
       <x:c r="F86" s="97" t="str"/>
+      <x:c r="G86" s="97" t="str"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="97" t="str">
@@ -2944,6 +3034,7 @@
       </x:c>
       <x:c r="E87" s="97" t="str"/>
       <x:c r="F87" s="97" t="str"/>
+      <x:c r="G87" s="97" t="str"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="97" t="str">
@@ -2960,6 +3051,7 @@
       </x:c>
       <x:c r="E88" s="97" t="str"/>
       <x:c r="F88" s="97" t="str"/>
+      <x:c r="G88" s="97" t="str"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="97" t="str">
@@ -2976,6 +3068,7 @@
       </x:c>
       <x:c r="E89" s="97" t="str"/>
       <x:c r="F89" s="97" t="str"/>
+      <x:c r="G89" s="97" t="str"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="97" t="str">
@@ -2992,6 +3085,7 @@
       </x:c>
       <x:c r="E90" s="97" t="str"/>
       <x:c r="F90" s="97" t="str"/>
+      <x:c r="G90" s="97" t="str"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="97" t="str">
@@ -3008,6 +3102,7 @@
       </x:c>
       <x:c r="E91" s="97" t="str"/>
       <x:c r="F91" s="97" t="str"/>
+      <x:c r="G91" s="97" t="str"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="97" t="str">
@@ -3024,6 +3119,7 @@
       </x:c>
       <x:c r="E92" s="97" t="str"/>
       <x:c r="F92" s="97" t="str"/>
+      <x:c r="G92" s="97" t="str"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="97" t="str">
@@ -3038,6 +3134,7 @@
       </x:c>
       <x:c r="E93" s="97" t="str"/>
       <x:c r="F93" s="97" t="str"/>
+      <x:c r="G93" s="97" t="str"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="97" t="str">
@@ -3052,10 +3149,11 @@
       <x:c r="D94" s="97" t="str">
         <x:v>I180;I181;I182</x:v>
       </x:c>
-      <x:c r="E94" s="97" t="str">
+      <x:c r="E94" s="97" t="str"/>
+      <x:c r="F94" s="97" t="str">
         <x:v>James is the corrected third child name; earlier draft said Janet.</x:v>
       </x:c>
-      <x:c r="F94" s="97" t="str"/>
+      <x:c r="G94" s="97" t="str"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="97" t="str">
@@ -3072,6 +3170,7 @@
       </x:c>
       <x:c r="E95" s="97" t="str"/>
       <x:c r="F95" s="97" t="str"/>
+      <x:c r="G95" s="97" t="str"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="97" t="str">
@@ -3086,10 +3185,11 @@
       <x:c r="D96" s="97" t="str">
         <x:v>I001;I175</x:v>
       </x:c>
-      <x:c r="E96" s="97" t="str">
+      <x:c r="E96" s="97" t="str"/>
+      <x:c r="F96" s="97" t="str">
         <x:v>Jan is Fredric and Arianna's biological mother; Henry is recorded as their father in the recovered canonical package.</x:v>
       </x:c>
-      <x:c r="F96" s="97" t="str">
+      <x:c r="G96" s="97" t="str">
         <x:v>S28</x:v>
       </x:c>
     </x:row>
@@ -3108,6 +3208,7 @@
       </x:c>
       <x:c r="E97" s="97" t="str"/>
       <x:c r="F97" s="97" t="str"/>
+      <x:c r="G97" s="97" t="str"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="97" t="str">
@@ -3122,10 +3223,11 @@
       <x:c r="D98" s="97" t="str">
         <x:v>I204;I205</x:v>
       </x:c>
-      <x:c r="E98" s="97" t="str">
+      <x:c r="E98" s="97" t="str"/>
+      <x:c r="F98" s="97" t="str">
         <x:v>Carey is the one and only daughter; Mark is the other child.</x:v>
       </x:c>
-      <x:c r="F98" s="97" t="str"/>
+      <x:c r="G98" s="97" t="str"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="97" t="str">
@@ -3138,10 +3240,11 @@
         <x:v>I185</x:v>
       </x:c>
       <x:c r="D99" s="97" t="str"/>
-      <x:c r="E99" s="97" t="str">
+      <x:c r="E99" s="97" t="str"/>
+      <x:c r="F99" s="97" t="str">
         <x:v>Dave and Kathy Werblo</x:v>
       </x:c>
-      <x:c r="F99" s="97" t="str"/>
+      <x:c r="G99" s="97" t="str"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="97" t="str">
@@ -3154,10 +3257,11 @@
         <x:v>I188</x:v>
       </x:c>
       <x:c r="D100" s="97" t="str"/>
-      <x:c r="E100" s="97" t="str">
+      <x:c r="E100" s="97" t="str"/>
+      <x:c r="F100" s="97" t="str">
         <x:v>John and Celeste</x:v>
       </x:c>
-      <x:c r="F100" s="97" t="str"/>
+      <x:c r="G100" s="97" t="str"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="97" t="str">
@@ -3170,10 +3274,11 @@
         <x:v>I189</x:v>
       </x:c>
       <x:c r="D101" s="97" t="str"/>
-      <x:c r="E101" s="97" t="str">
+      <x:c r="E101" s="97" t="str"/>
+      <x:c r="F101" s="97" t="str">
         <x:v>Gordon and Susan Galbraith</x:v>
       </x:c>
-      <x:c r="F101" s="97" t="str"/>
+      <x:c r="G101" s="97" t="str"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="97" t="str">
@@ -3186,10 +3291,11 @@
         <x:v>I191</x:v>
       </x:c>
       <x:c r="D102" s="97" t="str"/>
-      <x:c r="E102" s="97" t="str">
+      <x:c r="E102" s="97" t="str"/>
+      <x:c r="F102" s="97" t="str">
         <x:v>Historical spouse shown in 1998 chart</x:v>
       </x:c>
-      <x:c r="F102" s="97" t="str"/>
+      <x:c r="G102" s="97" t="str"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="97" t="str">
@@ -3202,10 +3308,11 @@
         <x:v>I195</x:v>
       </x:c>
       <x:c r="D103" s="97" t="str"/>
-      <x:c r="E103" s="97" t="str">
+      <x:c r="E103" s="97" t="str"/>
+      <x:c r="F103" s="97" t="str">
         <x:v>John and Sandy Hill</x:v>
       </x:c>
-      <x:c r="F103" s="97" t="str"/>
+      <x:c r="G103" s="97" t="str"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="97" t="str">
@@ -3218,10 +3325,11 @@
         <x:v>I198</x:v>
       </x:c>
       <x:c r="D104" s="97" t="str"/>
-      <x:c r="E104" s="97" t="str">
+      <x:c r="E104" s="97" t="str"/>
+      <x:c r="F104" s="97" t="str">
         <x:v>Ross and Carrie McCormick</x:v>
       </x:c>
-      <x:c r="F104" s="97" t="str"/>
+      <x:c r="G104" s="97" t="str"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="97" t="str">
@@ -3234,10 +3342,11 @@
         <x:v>I201</x:v>
       </x:c>
       <x:c r="D105" s="97" t="str"/>
-      <x:c r="E105" s="97" t="str">
+      <x:c r="E105" s="97" t="str"/>
+      <x:c r="F105" s="97" t="str">
         <x:v>Charles and Judy McCormick</x:v>
       </x:c>
-      <x:c r="F105" s="97" t="str"/>
+      <x:c r="G105" s="97" t="str"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="97" t="str">
@@ -3252,10 +3361,11 @@
       <x:c r="D106" s="97" t="str">
         <x:v>I176;I269</x:v>
       </x:c>
-      <x:c r="E106" s="97" t="str">
+      <x:c r="E106" s="97" t="str"/>
+      <x:c r="F106" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package. | Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F106" s="97" t="str">
+      <x:c r="G106" s="97" t="str">
         <x:v>S26;S27</x:v>
       </x:c>
     </x:row>
@@ -3272,10 +3382,11 @@
       <x:c r="D107" s="97" t="str">
         <x:v>I207;I270</x:v>
       </x:c>
-      <x:c r="E107" s="97" t="str">
+      <x:c r="E107" s="97" t="str"/>
+      <x:c r="F107" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package. | Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F107" s="97" t="str">
+      <x:c r="G107" s="97" t="str">
         <x:v>S26;S27</x:v>
       </x:c>
     </x:row>
@@ -3292,10 +3403,11 @@
       <x:c r="D108" s="97" t="str">
         <x:v>I208;I282</x:v>
       </x:c>
-      <x:c r="E108" s="97" t="str">
+      <x:c r="E108" s="97" t="str"/>
+      <x:c r="F108" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package. | Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F108" s="97" t="str">
+      <x:c r="G108" s="97" t="str">
         <x:v>S26;S27</x:v>
       </x:c>
     </x:row>
@@ -3312,10 +3424,11 @@
       <x:c r="D109" s="97" t="str">
         <x:v>I211</x:v>
       </x:c>
-      <x:c r="E109" s="97" t="str">
+      <x:c r="E109" s="97" t="str"/>
+      <x:c r="F109" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F109" s="97" t="str">
+      <x:c r="G109" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3332,10 +3445,11 @@
       <x:c r="D110" s="97" t="str">
         <x:v>I212</x:v>
       </x:c>
-      <x:c r="E110" s="97" t="str">
+      <x:c r="E110" s="97" t="str"/>
+      <x:c r="F110" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F110" s="97" t="str">
+      <x:c r="G110" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3352,10 +3466,11 @@
       <x:c r="D111" s="97" t="str">
         <x:v>I213</x:v>
       </x:c>
-      <x:c r="E111" s="97" t="str">
+      <x:c r="E111" s="97" t="str"/>
+      <x:c r="F111" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F111" s="97" t="str">
+      <x:c r="G111" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3372,10 +3487,11 @@
       <x:c r="D112" s="97" t="str">
         <x:v>I218;I274;I277</x:v>
       </x:c>
-      <x:c r="E112" s="97" t="str">
+      <x:c r="E112" s="97" t="str"/>
+      <x:c r="F112" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package. | Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F112" s="97" t="str">
+      <x:c r="G112" s="97" t="str">
         <x:v>S26;S27</x:v>
       </x:c>
     </x:row>
@@ -3392,10 +3508,11 @@
       <x:c r="D113" s="97" t="str">
         <x:v>I219;I283</x:v>
       </x:c>
-      <x:c r="E113" s="97" t="str">
+      <x:c r="E113" s="97" t="str"/>
+      <x:c r="F113" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package. | Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F113" s="97" t="str">
+      <x:c r="G113" s="97" t="str">
         <x:v>S26;S27</x:v>
       </x:c>
     </x:row>
@@ -3412,10 +3529,11 @@
       <x:c r="D114" s="97" t="str">
         <x:v>I220</x:v>
       </x:c>
-      <x:c r="E114" s="97" t="str">
+      <x:c r="E114" s="97" t="str"/>
+      <x:c r="F114" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F114" s="97" t="str">
+      <x:c r="G114" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3432,10 +3550,11 @@
       <x:c r="D115" s="97" t="str">
         <x:v>I222</x:v>
       </x:c>
-      <x:c r="E115" s="97" t="str">
+      <x:c r="E115" s="97" t="str"/>
+      <x:c r="F115" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F115" s="97" t="str">
+      <x:c r="G115" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3452,10 +3571,11 @@
       <x:c r="D116" s="97" t="str">
         <x:v>I223</x:v>
       </x:c>
-      <x:c r="E116" s="97" t="str">
+      <x:c r="E116" s="97" t="str"/>
+      <x:c r="F116" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F116" s="97" t="str">
+      <x:c r="G116" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3472,10 +3592,11 @@
       <x:c r="D117" s="97" t="str">
         <x:v>I225</x:v>
       </x:c>
-      <x:c r="E117" s="97" t="str">
+      <x:c r="E117" s="97" t="str"/>
+      <x:c r="F117" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F117" s="97" t="str">
+      <x:c r="G117" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3492,10 +3613,11 @@
       <x:c r="D118" s="97" t="str">
         <x:v>I227</x:v>
       </x:c>
-      <x:c r="E118" s="97" t="str">
+      <x:c r="E118" s="97" t="str"/>
+      <x:c r="F118" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F118" s="97" t="str">
+      <x:c r="G118" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3512,10 +3634,11 @@
       <x:c r="D119" s="97" t="str">
         <x:v>I228</x:v>
       </x:c>
-      <x:c r="E119" s="97" t="str">
+      <x:c r="E119" s="97" t="str"/>
+      <x:c r="F119" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F119" s="97" t="str">
+      <x:c r="G119" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3532,10 +3655,11 @@
       <x:c r="D120" s="97" t="str">
         <x:v>I229</x:v>
       </x:c>
-      <x:c r="E120" s="97" t="str">
+      <x:c r="E120" s="97" t="str"/>
+      <x:c r="F120" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F120" s="97" t="str">
+      <x:c r="G120" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3552,10 +3676,11 @@
       <x:c r="D121" s="97" t="str">
         <x:v>I235</x:v>
       </x:c>
-      <x:c r="E121" s="97" t="str">
+      <x:c r="E121" s="97" t="str"/>
+      <x:c r="F121" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F121" s="97" t="str">
+      <x:c r="G121" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3570,10 +3695,11 @@
       <x:c r="D122" s="97" t="str">
         <x:v>I236</x:v>
       </x:c>
-      <x:c r="E122" s="97" t="str">
+      <x:c r="E122" s="97" t="str"/>
+      <x:c r="F122" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F122" s="97" t="str">
+      <x:c r="G122" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3590,10 +3716,11 @@
       <x:c r="D123" s="97" t="str">
         <x:v>I238</x:v>
       </x:c>
-      <x:c r="E123" s="97" t="str">
+      <x:c r="E123" s="97" t="str"/>
+      <x:c r="F123" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F123" s="97" t="str">
+      <x:c r="G123" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3610,10 +3737,11 @@
       <x:c r="D124" s="97" t="str">
         <x:v>I239</x:v>
       </x:c>
-      <x:c r="E124" s="97" t="str">
+      <x:c r="E124" s="97" t="str"/>
+      <x:c r="F124" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F124" s="97" t="str">
+      <x:c r="G124" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3630,10 +3758,11 @@
       <x:c r="D125" s="97" t="str">
         <x:v>I240</x:v>
       </x:c>
-      <x:c r="E125" s="97" t="str">
+      <x:c r="E125" s="97" t="str"/>
+      <x:c r="F125" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F125" s="97" t="str">
+      <x:c r="G125" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3650,10 +3779,11 @@
       <x:c r="D126" s="97" t="str">
         <x:v>I241</x:v>
       </x:c>
-      <x:c r="E126" s="97" t="str">
+      <x:c r="E126" s="97" t="str"/>
+      <x:c r="F126" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F126" s="97" t="str">
+      <x:c r="G126" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3670,10 +3800,11 @@
       <x:c r="D127" s="97" t="str">
         <x:v>I245</x:v>
       </x:c>
-      <x:c r="E127" s="97" t="str">
+      <x:c r="E127" s="97" t="str"/>
+      <x:c r="F127" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F127" s="97" t="str">
+      <x:c r="G127" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3690,10 +3821,11 @@
       <x:c r="D128" s="97" t="str">
         <x:v>I246</x:v>
       </x:c>
-      <x:c r="E128" s="97" t="str">
+      <x:c r="E128" s="97" t="str"/>
+      <x:c r="F128" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F128" s="97" t="str">
+      <x:c r="G128" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3710,10 +3842,11 @@
       <x:c r="D129" s="97" t="str">
         <x:v>I247</x:v>
       </x:c>
-      <x:c r="E129" s="97" t="str">
+      <x:c r="E129" s="97" t="str"/>
+      <x:c r="F129" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F129" s="97" t="str">
+      <x:c r="G129" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3730,10 +3863,11 @@
       <x:c r="D130" s="97" t="str">
         <x:v>I248</x:v>
       </x:c>
-      <x:c r="E130" s="97" t="str">
+      <x:c r="E130" s="97" t="str"/>
+      <x:c r="F130" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F130" s="97" t="str">
+      <x:c r="G130" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3750,10 +3884,11 @@
       <x:c r="D131" s="97" t="str">
         <x:v>I249</x:v>
       </x:c>
-      <x:c r="E131" s="97" t="str">
+      <x:c r="E131" s="97" t="str"/>
+      <x:c r="F131" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F131" s="97" t="str">
+      <x:c r="G131" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3770,10 +3905,11 @@
       <x:c r="D132" s="97" t="str">
         <x:v>I250</x:v>
       </x:c>
-      <x:c r="E132" s="97" t="str">
+      <x:c r="E132" s="97" t="str"/>
+      <x:c r="F132" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F132" s="97" t="str">
+      <x:c r="G132" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3790,10 +3926,11 @@
       <x:c r="D133" s="97" t="str">
         <x:v>I251</x:v>
       </x:c>
-      <x:c r="E133" s="97" t="str">
+      <x:c r="E133" s="97" t="str"/>
+      <x:c r="F133" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F133" s="97" t="str">
+      <x:c r="G133" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3808,10 +3945,11 @@
       <x:c r="D134" s="97" t="str">
         <x:v>I254</x:v>
       </x:c>
-      <x:c r="E134" s="97" t="str">
+      <x:c r="E134" s="97" t="str"/>
+      <x:c r="F134" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F134" s="97" t="str">
+      <x:c r="G134" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3828,10 +3966,11 @@
       <x:c r="D135" s="97" t="str">
         <x:v>I261</x:v>
       </x:c>
-      <x:c r="E135" s="97" t="str">
+      <x:c r="E135" s="97" t="str"/>
+      <x:c r="F135" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F135" s="97" t="str">
+      <x:c r="G135" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3848,10 +3987,11 @@
       <x:c r="D136" s="97" t="str">
         <x:v>I264;I284;I285;I294</x:v>
       </x:c>
-      <x:c r="E136" s="97" t="str">
+      <x:c r="E136" s="97" t="str"/>
+      <x:c r="F136" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package. | Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F136" s="97" t="str">
+      <x:c r="G136" s="97" t="str">
         <x:v>S26;S27</x:v>
       </x:c>
     </x:row>
@@ -3868,10 +4008,11 @@
       <x:c r="D137" s="97" t="str">
         <x:v>I265</x:v>
       </x:c>
-      <x:c r="E137" s="97" t="str">
+      <x:c r="E137" s="97" t="str"/>
+      <x:c r="F137" s="97" t="str">
         <x:v>Relationship merged from the records-first Vollmer-Marsh research package.</x:v>
       </x:c>
-      <x:c r="F137" s="97" t="str">
+      <x:c r="G137" s="97" t="str">
         <x:v>S26</x:v>
       </x:c>
     </x:row>
@@ -3888,10 +4029,11 @@
       <x:c r="D138" s="97" t="str">
         <x:v>I272;I273</x:v>
       </x:c>
-      <x:c r="E138" s="97" t="str">
+      <x:c r="E138" s="97" t="str"/>
+      <x:c r="F138" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F138" s="97" t="str">
+      <x:c r="G138" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -3908,10 +4050,11 @@
       <x:c r="D139" s="97" t="str">
         <x:v>I276</x:v>
       </x:c>
-      <x:c r="E139" s="97" t="str">
+      <x:c r="E139" s="97" t="str"/>
+      <x:c r="F139" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F139" s="97" t="str">
+      <x:c r="G139" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -3928,10 +4071,11 @@
       <x:c r="D140" s="97" t="str">
         <x:v>I279;I280;I281</x:v>
       </x:c>
-      <x:c r="E140" s="97" t="str">
+      <x:c r="E140" s="97" t="str"/>
+      <x:c r="F140" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F140" s="97" t="str">
+      <x:c r="G140" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -3948,10 +4092,11 @@
       <x:c r="D141" s="97" t="str">
         <x:v>I287;I288;I289;I290;I291;I292;I293</x:v>
       </x:c>
-      <x:c r="E141" s="97" t="str">
+      <x:c r="E141" s="97" t="str"/>
+      <x:c r="F141" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F141" s="97" t="str">
+      <x:c r="G141" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -3968,10 +4113,11 @@
       <x:c r="D142" s="97" t="str">
         <x:v>I317</x:v>
       </x:c>
-      <x:c r="E142" s="97" t="str">
+      <x:c r="E142" s="97" t="str"/>
+      <x:c r="F142" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F142" s="97" t="str">
+      <x:c r="G142" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -3988,10 +4134,11 @@
       <x:c r="D143" s="97" t="str">
         <x:v>I322;I323</x:v>
       </x:c>
-      <x:c r="E143" s="97" t="str">
+      <x:c r="E143" s="97" t="str"/>
+      <x:c r="F143" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F143" s="97" t="str">
+      <x:c r="G143" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -4008,10 +4155,11 @@
       <x:c r="D144" s="97" t="str">
         <x:v>I331</x:v>
       </x:c>
-      <x:c r="E144" s="97" t="str">
+      <x:c r="E144" s="97" t="str"/>
+      <x:c r="F144" s="97" t="str">
         <x:v>Collateral relationship merged from the extended-family research package.</x:v>
       </x:c>
-      <x:c r="F144" s="97" t="str">
+      <x:c r="G144" s="97" t="str">
         <x:v>S27</x:v>
       </x:c>
     </x:row>
@@ -4026,17 +4174,62 @@
       <x:c r="D145" s="97" t="str">
         <x:v>I335</x:v>
       </x:c>
-      <x:c r="E145" s="97" t="str">
+      <x:c r="E145" s="97" t="str"/>
+      <x:c r="F145" s="97" t="str">
         <x:v>Chris's father was not confirmed and is intentionally omitted.</x:v>
       </x:c>
-      <x:c r="F145" s="97" t="str">
+      <x:c r="G145" s="97" t="str">
         <x:v>S28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="97" t="str">
+        <x:v>F145</x:v>
+      </x:c>
+      <x:c r="B146" s="97" t="str">
+        <x:v>I336</x:v>
+      </x:c>
+      <x:c r="C146" s="97" t="str">
+        <x:v>I337</x:v>
+      </x:c>
+      <x:c r="D146" s="97" t="str">
+        <x:v>I334</x:v>
+      </x:c>
+      <x:c r="E146" s="97" t="str">
+        <x:v>16 NOV 1929; Pierce County, Washington</x:v>
+      </x:c>
+      <x:c r="F146" s="97" t="str">
+        <x:v>The 1950 census identifies Mary Alice as William and Alice's daughter.</x:v>
+      </x:c>
+      <x:c r="G146" s="97" t="str">
+        <x:v>S32;S33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="97" t="str">
+        <x:v>F146</x:v>
+      </x:c>
+      <x:c r="B147" s="97" t="str">
+        <x:v>I176</x:v>
+      </x:c>
+      <x:c r="C147" s="97" t="str">
+        <x:v>I334</x:v>
+      </x:c>
+      <x:c r="D147" s="97" t="str"/>
+      <x:c r="E147" s="97" t="str">
+        <x:v>16 SEP 1955; King County, Washington</x:v>
+      </x:c>
+      <x:c r="F147" s="97" t="str">
+        <x:v>Owner-confirmed first marriage of Henry, before his marriage to Jan. This spouse link does not establish Chris's father.</x:v>
+      </x:c>
+      <x:c r="G147" s="97" t="str">
+        <x:v>S28;S31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R814fb72d9ad448e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42c39c52c2cb4e0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4514,16 +4707,16 @@
         <x:v>S28</x:v>
       </x:c>
       <x:c r="B29" s="97" t="str">
-        <x:v>Owner statements on Jan Muller Vollmer, Mary Alice, and Chris Vollmer</x:v>
+        <x:v>Owner statements on Jan Muller Vollmer, Mary Alice Thoren, William Thoren, and Chris Vollmer</x:v>
       </x:c>
       <x:c r="C29" s="97" t="str">
         <x:v>Fredric Muller Vollmer</x:v>
       </x:c>
       <x:c r="D29" s="97" t="str">
-        <x:v>1 SEP 2026</x:v>
+        <x:v>2 SEP 2026</x:v>
       </x:c>
       <x:c r="E29" s="97" t="str">
-        <x:v>Jan is Fredric's biological mother; Mary Alice is Chris Vollmer's mother; Jan is Chris's stepmother. Chris's father was not stated.</x:v>
+        <x:v>Jan is Fredric's biological mother; Mary Alice Thoren was born in Port Townsend, was Henry's first wife, and is Chris Vollmer's mother; Jan is Chris's stepmother. William 'Bill' Thoren was remembered as Mary Alice's father. Chris's father was not stated.</x:v>
       </x:c>
       <x:c r="F29" s="97" t="str">
         <x:v>cross-chat consolidation</x:v>
@@ -4571,63 +4764,75 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="97" t="str">
-        <x:v>RECORD-1648-06-15_deborah-hopkins_birth-register</x:v>
+        <x:v>S31</x:v>
       </x:c>
       <x:c r="B32" s="97" t="str">
-        <x:v>1648-06-15_deborah-hopkins_birth-register.jpg</x:v>
-      </x:c>
-      <x:c r="C32" s="97" t="str"/>
-      <x:c r="D32" s="97" t="str"/>
+        <x:v>Henry R Vollmer and Mary A Thoren marriage record</x:v>
+      </x:c>
+      <x:c r="C32" s="97" t="str">
+        <x:v>Washington State Archives; King County Auditor</x:v>
+      </x:c>
+      <x:c r="D32" s="97" t="str">
+        <x:v>16 SEP 1955</x:v>
+      </x:c>
       <x:c r="E32" s="97" t="str">
-        <x:v>4e6dd607655f9c2b251e3974596d63276178e76761116b370a8b16e0219f3f98</x:v>
+        <x:v>King County Marriage Records, 1855-2017; reference kingcoarchmc207309; https://digitalarchives.wa.gov/Record/View/437A4FBD9EF3DA4BD90C60795808BC69</x:v>
       </x:c>
       <x:c r="F32" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="97" t="str">
-        <x:v>RECORD-1667-02-05_ephraim-doane_mary-knowles_marriage-register</x:v>
+        <x:v>S32</x:v>
       </x:c>
       <x:c r="B33" s="97" t="str">
-        <x:v>1667-02-05_ephraim-doane_mary-knowles_marriage-register.jpg</x:v>
-      </x:c>
-      <x:c r="C33" s="97" t="str"/>
-      <x:c r="D33" s="97" t="str"/>
+        <x:v>1950 United States census household of William J Thoren</x:v>
+      </x:c>
+      <x:c r="C33" s="97" t="str">
+        <x:v>U.S. Census Bureau; National Archives and Records Administration</x:v>
+      </x:c>
+      <x:c r="D33" s="97" t="str">
+        <x:v>5 APR 1950</x:v>
+      </x:c>
       <x:c r="E33" s="97" t="str">
-        <x:v>89ae0910e197b39bd902ca52685d144ab55193a340c5e6d3dbeb15a811487faa</x:v>
+        <x:v>Seattle, King County, Washington, enumeration district 40-124, sheet 74, lines 23-25. William J Thoren, wife Alice, and daughter Mary Alice; NARA image 43290879-Washington-031283-0021; https://1950census.archives.gov/search/?ed=40-124&amp;state=WA&amp;page=1</x:v>
       </x:c>
       <x:c r="F33" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="97" t="str">
-        <x:v>RECORD-1682-02-04_joshua-cook_birth-register</x:v>
+        <x:v>S33</x:v>
       </x:c>
       <x:c r="B34" s="97" t="str">
-        <x:v>1682-02-04_joshua-cook_birth-register.jpg</x:v>
-      </x:c>
-      <x:c r="C34" s="97" t="str"/>
-      <x:c r="D34" s="97" t="str"/>
+        <x:v>William J Thoren and Alice Gallaher marriage record</x:v>
+      </x:c>
+      <x:c r="C34" s="97" t="str">
+        <x:v>Washington State Archives; Pierce County Auditor</x:v>
+      </x:c>
+      <x:c r="D34" s="97" t="str">
+        <x:v>16 NOV 1929</x:v>
+      </x:c>
       <x:c r="E34" s="97" t="str">
-        <x:v>726be1a255bf2abe13e2cdc2d149bcddf7dfb1702c466ab4e215d38133e9ea46</x:v>
+        <x:v>Pierce County Auditor Marriage Records, reference prcmc-v23-00709; https://digitalarchives.wa.gov/Record/View/33AF9C076D80A9452C66FD351D17CD73</x:v>
       </x:c>
       <x:c r="F34" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="97" t="str">
-        <x:v>RECORD-1682-04_patience-doane_birth-register</x:v>
+        <x:v>RECORD-1648-06-15_deborah-hopkins_birth-register</x:v>
       </x:c>
       <x:c r="B35" s="97" t="str">
-        <x:v>1682-04_patience-doane_birth-register.jpg</x:v>
+        <x:v>1648-06-15_deborah-hopkins_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C35" s="97" t="str"/>
       <x:c r="D35" s="97" t="str"/>
       <x:c r="E35" s="97" t="str">
-        <x:v>c754af467f7252cd6952af7bc5948ce2ca5f77fdb7c7e60a6941088448c32e4a</x:v>
+        <x:v>4e6dd607655f9c2b251e3974596d63276178e76761116b370a8b16e0219f3f98</x:v>
       </x:c>
       <x:c r="F35" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4635,15 +4840,15 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="97" t="str">
-        <x:v>RECORD-1696_joshua-lane_birth-record</x:v>
+        <x:v>RECORD-1667-02-05_ephraim-doane_mary-knowles_marriage-register</x:v>
       </x:c>
       <x:c r="B36" s="97" t="str">
-        <x:v>1696_joshua-lane_birth-record.jpg</x:v>
+        <x:v>1667-02-05_ephraim-doane_mary-knowles_marriage-register.jpg</x:v>
       </x:c>
       <x:c r="C36" s="97" t="str"/>
       <x:c r="D36" s="97" t="str"/>
       <x:c r="E36" s="97" t="str">
-        <x:v>23c17bccf0b93d5ca970ddc6458dc14f264e129c5650c13a9e613dc57e94371e</x:v>
+        <x:v>89ae0910e197b39bd902ca52685d144ab55193a340c5e6d3dbeb15a811487faa</x:v>
       </x:c>
       <x:c r="F36" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4651,15 +4856,15 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="97" t="str">
-        <x:v>RECORD-1717_joshua-lane_bathsheba-robie_marriage-record</x:v>
+        <x:v>RECORD-1682-02-04_joshua-cook_birth-register</x:v>
       </x:c>
       <x:c r="B37" s="97" t="str">
-        <x:v>1717_joshua-lane_bathsheba-robie_marriage-record.jpg</x:v>
+        <x:v>1682-02-04_joshua-cook_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C37" s="97" t="str"/>
       <x:c r="D37" s="97" t="str"/>
       <x:c r="E37" s="97" t="str">
-        <x:v>15e63b00090b98e21bb4ae4d28cc0d2a620bbe75946c63efe681f5b512fb6b9c</x:v>
+        <x:v>726be1a255bf2abe13e2cdc2d149bcddf7dfb1702c466ab4e215d38133e9ea46</x:v>
       </x:c>
       <x:c r="F37" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4667,15 +4872,15 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="97" t="str">
-        <x:v>RECORD-1718_samuel-lane_birth-record</x:v>
+        <x:v>RECORD-1682-04_patience-doane_birth-register</x:v>
       </x:c>
       <x:c r="B38" s="97" t="str">
-        <x:v>1718_samuel-lane_birth-record.jpg</x:v>
+        <x:v>1682-04_patience-doane_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C38" s="97" t="str"/>
       <x:c r="D38" s="97" t="str"/>
       <x:c r="E38" s="97" t="str">
-        <x:v>0200f2252b3392cf2fa2ecb3d58b9ddef31b998ce5d76ef552bfab2ee7eda016</x:v>
+        <x:v>c754af467f7252cd6952af7bc5948ce2ca5f77fdb7c7e60a6941088448c32e4a</x:v>
       </x:c>
       <x:c r="F38" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4683,15 +4888,15 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="97" t="str">
-        <x:v>RECORD-1722_mary-james_birth-record</x:v>
+        <x:v>RECORD-1696_joshua-lane_birth-record</x:v>
       </x:c>
       <x:c r="B39" s="97" t="str">
-        <x:v>1722_mary-james_birth-record.jpg</x:v>
+        <x:v>1696_joshua-lane_birth-record.jpg</x:v>
       </x:c>
       <x:c r="C39" s="97" t="str"/>
       <x:c r="D39" s="97" t="str"/>
       <x:c r="E39" s="97" t="str">
-        <x:v>189899f04cbc5dc801896487041938515771118dabdb1af87ed6662a4f6ffcd9</x:v>
+        <x:v>23c17bccf0b93d5ca970ddc6458dc14f264e129c5650c13a9e613dc57e94371e</x:v>
       </x:c>
       <x:c r="F39" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4699,15 +4904,15 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="97" t="str">
-        <x:v>RECORD-1741-12-24_samuel-lane_mary-james_marriage</x:v>
+        <x:v>RECORD-1717_joshua-lane_bathsheba-robie_marriage-record</x:v>
       </x:c>
       <x:c r="B40" s="97" t="str">
-        <x:v>1741-12-24_samuel-lane_mary-james_marriage.jpg</x:v>
+        <x:v>1717_joshua-lane_bathsheba-robie_marriage-record.jpg</x:v>
       </x:c>
       <x:c r="C40" s="97" t="str"/>
       <x:c r="D40" s="97" t="str"/>
       <x:c r="E40" s="97" t="str">
-        <x:v>fd6d017aaaa9f3c51bd77b7c6a0a007e08a6b28b3eacd4323314c75ced5f61b4</x:v>
+        <x:v>15e63b00090b98e21bb4ae4d28cc0d2a620bbe75946c63efe681f5b512fb6b9c</x:v>
       </x:c>
       <x:c r="F40" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4715,15 +4920,15 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="97" t="str">
-        <x:v>RECORD-1748-02-09_joshua-lane_nh-birth</x:v>
+        <x:v>RECORD-1718_samuel-lane_birth-record</x:v>
       </x:c>
       <x:c r="B41" s="97" t="str">
-        <x:v>1748-02-09_joshua-lane_nh-birth.jpg</x:v>
+        <x:v>1718_samuel-lane_birth-record.jpg</x:v>
       </x:c>
       <x:c r="C41" s="97" t="str"/>
       <x:c r="D41" s="97" t="str"/>
       <x:c r="E41" s="97" t="str">
-        <x:v>8b75cc1094090d59c00e82213eddedaf9393a4953d2ae2703bcc6fafbe5fa72b</x:v>
+        <x:v>0200f2252b3392cf2fa2ecb3d58b9ddef31b998ce5d76ef552bfab2ee7eda016</x:v>
       </x:c>
       <x:c r="F41" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4731,15 +4936,15 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="97" t="str">
-        <x:v>RECORD-1769-11-15_joshua-lane_hannah-tilton_marriage</x:v>
+        <x:v>RECORD-1722_mary-james_birth-record</x:v>
       </x:c>
       <x:c r="B42" s="97" t="str">
-        <x:v>1769-11-15_joshua-lane_hannah-tilton_marriage.jpg</x:v>
+        <x:v>1722_mary-james_birth-record.jpg</x:v>
       </x:c>
       <x:c r="C42" s="97" t="str"/>
       <x:c r="D42" s="97" t="str"/>
       <x:c r="E42" s="97" t="str">
-        <x:v>9d1f204134ed96a42e5c7ddfe10e1265e03ae8c7af976cc6723f3836c6037d3e</x:v>
+        <x:v>189899f04cbc5dc801896487041938515771118dabdb1af87ed6662a4f6ffcd9</x:v>
       </x:c>
       <x:c r="F42" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4747,15 +4952,15 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="97" t="str">
-        <x:v>RECORD-1771-12-08_stephen-lane_nh-birth</x:v>
+        <x:v>RECORD-1741-12-24_samuel-lane_mary-james_marriage</x:v>
       </x:c>
       <x:c r="B43" s="97" t="str">
-        <x:v>1771-12-08_stephen-lane_nh-birth.jpg</x:v>
+        <x:v>1741-12-24_samuel-lane_mary-james_marriage.jpg</x:v>
       </x:c>
       <x:c r="C43" s="97" t="str"/>
       <x:c r="D43" s="97" t="str"/>
       <x:c r="E43" s="97" t="str">
-        <x:v>4e983a0346e7c1b3d08b50d78c339d06a10d4ba9e23b8d7a2c932aa69343fd72</x:v>
+        <x:v>fd6d017aaaa9f3c51bd77b7c6a0a007e08a6b28b3eacd4323314c75ced5f61b4</x:v>
       </x:c>
       <x:c r="F43" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4763,15 +4968,15 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="97" t="str">
-        <x:v>RECORD-1774-02-26_levi-cook_birth-register</x:v>
+        <x:v>RECORD-1748-02-09_joshua-lane_nh-birth</x:v>
       </x:c>
       <x:c r="B44" s="97" t="str">
-        <x:v>1774-02-26_levi-cook_birth-register.jpg</x:v>
+        <x:v>1748-02-09_joshua-lane_nh-birth.jpg</x:v>
       </x:c>
       <x:c r="C44" s="97" t="str"/>
       <x:c r="D44" s="97" t="str"/>
       <x:c r="E44" s="97" t="str">
-        <x:v>da32fa229e920c36321196b78361e9ea6df2ae57d08d34cf81279f9f727c5e26</x:v>
+        <x:v>8b75cc1094090d59c00e82213eddedaf9393a4953d2ae2703bcc6fafbe5fa72b</x:v>
       </x:c>
       <x:c r="F44" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4779,15 +4984,15 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="97" t="str">
-        <x:v>RECORD-1779-01-07_betsey-brown_birth-register</x:v>
+        <x:v>RECORD-1769-11-15_joshua-lane_hannah-tilton_marriage</x:v>
       </x:c>
       <x:c r="B45" s="97" t="str">
-        <x:v>1779-01-07_betsey-brown_birth-register.jpg</x:v>
+        <x:v>1769-11-15_joshua-lane_hannah-tilton_marriage.jpg</x:v>
       </x:c>
       <x:c r="C45" s="97" t="str"/>
       <x:c r="D45" s="97" t="str"/>
       <x:c r="E45" s="97" t="str">
-        <x:v>c43c3675e73e795d5d4ef90d64e64e746f1f9da1cf41ea0f2bbcddd01b50bfba</x:v>
+        <x:v>9d1f204134ed96a42e5c7ddfe10e1265e03ae8c7af976cc6723f3836c6037d3e</x:v>
       </x:c>
       <x:c r="F45" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4795,15 +5000,15 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="97" t="str">
-        <x:v>RECORD-1794-07-24_levi-cook_betsey-brown_marriage-register</x:v>
+        <x:v>RECORD-1771-12-08_stephen-lane_nh-birth</x:v>
       </x:c>
       <x:c r="B46" s="97" t="str">
-        <x:v>1794-07-24_levi-cook_betsey-brown_marriage-register.jpg</x:v>
+        <x:v>1771-12-08_stephen-lane_nh-birth.jpg</x:v>
       </x:c>
       <x:c r="C46" s="97" t="str"/>
       <x:c r="D46" s="97" t="str"/>
       <x:c r="E46" s="97" t="str">
-        <x:v>f3faf328a3ca886129787a18975b1c4892c5a5ed6bac9bebe5d6d4eb867f379f</x:v>
+        <x:v>4e983a0346e7c1b3d08b50d78c339d06a10d4ba9e23b8d7a2c932aa69343fd72</x:v>
       </x:c>
       <x:c r="F46" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4811,15 +5016,15 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="97" t="str">
-        <x:v>RECORD-1797-06-05_stephen-lane_lois-currier_marriage</x:v>
+        <x:v>RECORD-1774-02-26_levi-cook_birth-register</x:v>
       </x:c>
       <x:c r="B47" s="97" t="str">
-        <x:v>1797-06-05_stephen-lane_lois-currier_marriage.jpg</x:v>
+        <x:v>1774-02-26_levi-cook_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C47" s="97" t="str"/>
       <x:c r="D47" s="97" t="str"/>
       <x:c r="E47" s="97" t="str">
-        <x:v>6dd9495e06654018e796489a805f91471bd33329204c0b5171ee5425a898b280</x:v>
+        <x:v>da32fa229e920c36321196b78361e9ea6df2ae57d08d34cf81279f9f727c5e26</x:v>
       </x:c>
       <x:c r="F47" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4827,15 +5032,15 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="97" t="str">
-        <x:v>RECORD-1807-02-03_mary-lane_nh-birth-card</x:v>
+        <x:v>RECORD-1779-01-07_betsey-brown_birth-register</x:v>
       </x:c>
       <x:c r="B48" s="97" t="str">
-        <x:v>1807-02-03_mary-lane_nh-birth-card.jpg</x:v>
+        <x:v>1779-01-07_betsey-brown_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C48" s="97" t="str"/>
       <x:c r="D48" s="97" t="str"/>
       <x:c r="E48" s="97" t="str">
-        <x:v>54e52adccc86fbb08e9fd36c8ad80efbb130eb34178bf7f4cae9bfe9fae15351</x:v>
+        <x:v>c43c3675e73e795d5d4ef90d64e64e746f1f9da1cf41ea0f2bbcddd01b50bfba</x:v>
       </x:c>
       <x:c r="F48" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4843,15 +5048,15 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="97" t="str">
-        <x:v>RECORD-1840-09-16_stephen-lane_will</x:v>
+        <x:v>RECORD-1794-07-24_levi-cook_betsey-brown_marriage-register</x:v>
       </x:c>
       <x:c r="B49" s="97" t="str">
-        <x:v>1840-09-16_stephen-lane_will.jpg</x:v>
+        <x:v>1794-07-24_levi-cook_betsey-brown_marriage-register.jpg</x:v>
       </x:c>
       <x:c r="C49" s="97" t="str"/>
       <x:c r="D49" s="97" t="str"/>
       <x:c r="E49" s="97" t="str">
-        <x:v>773c3a78efbeac6efc48f53d6d01f7556aade77197bb59cb85265cb67c5b4f99</x:v>
+        <x:v>f3faf328a3ca886129787a18975b1c4892c5a5ed6bac9bebe5d6d4eb867f379f</x:v>
       </x:c>
       <x:c r="F49" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4859,15 +5064,15 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="97" t="str">
-        <x:v>RECORD-1841-05-05_stephen-lane_probate-letters</x:v>
+        <x:v>RECORD-1797-06-05_stephen-lane_lois-currier_marriage</x:v>
       </x:c>
       <x:c r="B50" s="97" t="str">
-        <x:v>1841-05-05_stephen-lane_probate-letters.jpg</x:v>
+        <x:v>1797-06-05_stephen-lane_lois-currier_marriage.jpg</x:v>
       </x:c>
       <x:c r="C50" s="97" t="str"/>
       <x:c r="D50" s="97" t="str"/>
       <x:c r="E50" s="97" t="str">
-        <x:v>dca2ab0c7608fe5ca72e5d18e3bb9d920173d4535609fca51f115c9de62c2c04</x:v>
+        <x:v>6dd9495e06654018e796489a805f91471bd33329204c0b5171ee5425a898b280</x:v>
       </x:c>
       <x:c r="F50" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4875,15 +5080,15 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="97" t="str">
-        <x:v>RECORD-1846-10-30_levi-cook_will_genesee</x:v>
+        <x:v>RECORD-1807-02-03_mary-lane_nh-birth-card</x:v>
       </x:c>
       <x:c r="B51" s="97" t="str">
-        <x:v>1846-10-30_levi-cook_will_genesee.jpg</x:v>
+        <x:v>1807-02-03_mary-lane_nh-birth-card.jpg</x:v>
       </x:c>
       <x:c r="C51" s="97" t="str"/>
       <x:c r="D51" s="97" t="str"/>
       <x:c r="E51" s="97" t="str">
-        <x:v>ca99721390ba6f33558e3a0ce805f614dabed6ee6aab6dce762506bf16f00235</x:v>
+        <x:v>54e52adccc86fbb08e9fd36c8ad80efbb130eb34178bf7f4cae9bfe9fae15351</x:v>
       </x:c>
       <x:c r="F51" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4891,15 +5096,15 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="97" t="str">
-        <x:v>RECORD-1862_peter-william-mcnaughton_civil-war-town-register</x:v>
+        <x:v>RECORD-1840-09-16_stephen-lane_will</x:v>
       </x:c>
       <x:c r="B52" s="97" t="str">
-        <x:v>1862_peter-william-mcnaughton_civil-war-town-register.jpg</x:v>
+        <x:v>1840-09-16_stephen-lane_will.jpg</x:v>
       </x:c>
       <x:c r="C52" s="97" t="str"/>
       <x:c r="D52" s="97" t="str"/>
       <x:c r="E52" s="97" t="str">
-        <x:v>7e767cf4e9ce3792ea381e5dcea992eade9ac9d7e361eae2e6927ed41b52a9b4</x:v>
+        <x:v>773c3a78efbeac6efc48f53d6d01f7556aade77197bb59cb85265cb67c5b4f99</x:v>
       </x:c>
       <x:c r="F52" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4907,15 +5112,15 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="97" t="str">
-        <x:v>RECORD-1868_relief-mcnaughton_dependent-pension-numerical-index</x:v>
+        <x:v>RECORD-1841-05-05_stephen-lane_probate-letters</x:v>
       </x:c>
       <x:c r="B53" s="97" t="str">
-        <x:v>1868_relief-mcnaughton_dependent-pension-numerical-index.jpg</x:v>
+        <x:v>1841-05-05_stephen-lane_probate-letters.jpg</x:v>
       </x:c>
       <x:c r="C53" s="97" t="str"/>
       <x:c r="D53" s="97" t="str"/>
       <x:c r="E53" s="97" t="str">
-        <x:v>122349eb44bcbf808eaa9d841bec77cb9b433ff01d7b88dd9f862441a237ed6e</x:v>
+        <x:v>dca2ab0c7608fe5ca72e5d18e3bb9d920173d4535609fca51f115c9de62c2c04</x:v>
       </x:c>
       <x:c r="F53" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4923,15 +5128,15 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="97" t="str">
-        <x:v>RECORD-1882-08-21_henry-vollmer_arrival-main</x:v>
+        <x:v>RECORD-1846-10-30_levi-cook_will_genesee</x:v>
       </x:c>
       <x:c r="B54" s="97" t="str">
-        <x:v>1882-08-21_henry-vollmer_arrival-main.jpg</x:v>
+        <x:v>1846-10-30_levi-cook_will_genesee.jpg</x:v>
       </x:c>
       <x:c r="C54" s="97" t="str"/>
       <x:c r="D54" s="97" t="str"/>
       <x:c r="E54" s="97" t="str">
-        <x:v>319186b29241957f4be18e4f2c4d350679c5b0c36f6ee3330ba90a62dbca0b24</x:v>
+        <x:v>ca99721390ba6f33558e3a0ce805f614dabed6ee6aab6dce762506bf16f00235</x:v>
       </x:c>
       <x:c r="F54" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4939,15 +5144,15 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="97" t="str">
-        <x:v>RECORD-1882-08-21_vollmer-family_arrival-main_page-0289</x:v>
+        <x:v>RECORD-1862_peter-william-mcnaughton_civil-war-town-register</x:v>
       </x:c>
       <x:c r="B55" s="97" t="str">
-        <x:v>1882-08-21_vollmer-family_arrival-main_page-0289.jpg</x:v>
+        <x:v>1862_peter-william-mcnaughton_civil-war-town-register.jpg</x:v>
       </x:c>
       <x:c r="C55" s="97" t="str"/>
       <x:c r="D55" s="97" t="str"/>
       <x:c r="E55" s="97" t="str">
-        <x:v>747649d753285ae52234547090101c60660612500bc3132a35f57b13a0ce9e11</x:v>
+        <x:v>7e767cf4e9ce3792ea381e5dcea992eade9ac9d7e361eae2e6927ed41b52a9b4</x:v>
       </x:c>
       <x:c r="F55" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4955,15 +5160,15 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="97" t="str">
-        <x:v>RECORD-1883-08-12_themes-pepper_anna-stelling_marriage-certificate</x:v>
+        <x:v>RECORD-1868_relief-mcnaughton_dependent-pension-numerical-index</x:v>
       </x:c>
       <x:c r="B56" s="97" t="str">
-        <x:v>1883-08-12_themes-pepper_anna-stelling_marriage-certificate.pdf</x:v>
+        <x:v>1868_relief-mcnaughton_dependent-pension-numerical-index.jpg</x:v>
       </x:c>
       <x:c r="C56" s="97" t="str"/>
       <x:c r="D56" s="97" t="str"/>
       <x:c r="E56" s="97" t="str">
-        <x:v>2a89c49df0051c74dbc241741e7b75dbabeff093782428e3a3b82cd002de44bd</x:v>
+        <x:v>122349eb44bcbf808eaa9d841bec77cb9b433ff01d7b88dd9f862441a237ed6e</x:v>
       </x:c>
       <x:c r="F56" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4971,15 +5176,15 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="97" t="str">
-        <x:v>RECORD-1884-03-14_female-pepper_birth-certificate</x:v>
+        <x:v>RECORD-1882-08-21_henry-vollmer_arrival-main</x:v>
       </x:c>
       <x:c r="B57" s="97" t="str">
-        <x:v>1884-03-14_female-pepper_birth-certificate.pdf</x:v>
+        <x:v>1882-08-21_henry-vollmer_arrival-main.jpg</x:v>
       </x:c>
       <x:c r="C57" s="97" t="str"/>
       <x:c r="D57" s="97" t="str"/>
       <x:c r="E57" s="97" t="str">
-        <x:v>d457e8478154d51688ddd777101aee2501f89ef8f4515eab0a8cf431076d7180</x:v>
+        <x:v>319186b29241957f4be18e4f2c4d350679c5b0c36f6ee3330ba90a62dbca0b24</x:v>
       </x:c>
       <x:c r="F57" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -4987,15 +5192,15 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="97" t="str">
-        <x:v>RECORD-1892_henry-vollmer_ny-state-census</x:v>
+        <x:v>RECORD-1882-08-21_vollmer-family_arrival-main_page-0289</x:v>
       </x:c>
       <x:c r="B58" s="97" t="str">
-        <x:v>1892_henry-vollmer_ny-state-census.jpg</x:v>
+        <x:v>1882-08-21_vollmer-family_arrival-main_page-0289.jpg</x:v>
       </x:c>
       <x:c r="C58" s="97" t="str"/>
       <x:c r="D58" s="97" t="str"/>
       <x:c r="E58" s="97" t="str">
-        <x:v>480f9a9c4d79a918392467e6ebf758452a8d200ad3692cb7f436a4654d688421</x:v>
+        <x:v>747649d753285ae52234547090101c60660612500bc3132a35f57b13a0ce9e11</x:v>
       </x:c>
       <x:c r="F58" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5003,15 +5208,15 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="97" t="str">
-        <x:v>RECORD-1896_mary-a-mcnaughton_widow-pension-index</x:v>
+        <x:v>RECORD-1883-08-12_themes-pepper_anna-stelling_marriage-certificate</x:v>
       </x:c>
       <x:c r="B59" s="97" t="str">
-        <x:v>1896_mary-a-mcnaughton_widow-pension-index.jpg</x:v>
+        <x:v>1883-08-12_themes-pepper_anna-stelling_marriage-certificate.pdf</x:v>
       </x:c>
       <x:c r="C59" s="97" t="str"/>
       <x:c r="D59" s="97" t="str"/>
       <x:c r="E59" s="97" t="str">
-        <x:v>14d064d694dc478f36bb570e78e29368a0259693dfb7217c05975c508bd01db8</x:v>
+        <x:v>2a89c49df0051c74dbc241741e7b75dbabeff093782428e3a3b82cd002de44bd</x:v>
       </x:c>
       <x:c r="F59" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5019,15 +5224,15 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="97" t="str">
-        <x:v>RECORD-1901_mayflower-descendant-vol3_john-doane-will</x:v>
+        <x:v>RECORD-1884-03-14_female-pepper_birth-certificate</x:v>
       </x:c>
       <x:c r="B60" s="97" t="str">
-        <x:v>1901_mayflower-descendant-vol3_john-doane-will.pdf</x:v>
+        <x:v>1884-03-14_female-pepper_birth-certificate.pdf</x:v>
       </x:c>
       <x:c r="C60" s="97" t="str"/>
       <x:c r="D60" s="97" t="str"/>
       <x:c r="E60" s="97" t="str">
-        <x:v>4d7d359130d69d3db9e5ebdec3f22833c097c0e9dad4e5602047f370bd057518</x:v>
+        <x:v>d457e8478154d51688ddd777101aee2501f89ef8f4515eab0a8cf431076d7180</x:v>
       </x:c>
       <x:c r="F60" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5035,15 +5240,15 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="97" t="str">
-        <x:v>RECORD-1904_mayflower-descendant-vol6_eastham-vital-records</x:v>
+        <x:v>RECORD-1892_henry-vollmer_ny-state-census</x:v>
       </x:c>
       <x:c r="B61" s="97" t="str">
-        <x:v>1904_mayflower-descendant-vol6_eastham-vital-records.pdf</x:v>
+        <x:v>1892_henry-vollmer_ny-state-census.jpg</x:v>
       </x:c>
       <x:c r="C61" s="97" t="str"/>
       <x:c r="D61" s="97" t="str"/>
       <x:c r="E61" s="97" t="str">
-        <x:v>105a13412229bb5489c9e245faa82209405ec7199e5fe371dc17a09d1351ba3a</x:v>
+        <x:v>480f9a9c4d79a918392467e6ebf758452a8d200ad3692cb7f436a4654d688421</x:v>
       </x:c>
       <x:c r="F61" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5051,15 +5256,15 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="97" t="str">
-        <x:v>RECORD-1905-08-05_henry-jj-vollmer_marriage-certificate</x:v>
+        <x:v>RECORD-1896_mary-a-mcnaughton_widow-pension-index</x:v>
       </x:c>
       <x:c r="B62" s="97" t="str">
-        <x:v>1905-08-05_henry-jj-vollmer_marriage-certificate.pdf</x:v>
+        <x:v>1896_mary-a-mcnaughton_widow-pension-index.jpg</x:v>
       </x:c>
       <x:c r="C62" s="97" t="str"/>
       <x:c r="D62" s="97" t="str"/>
       <x:c r="E62" s="97" t="str">
-        <x:v>59b537c81462fcba56c9827e5a015dacefafd451442735b8db6a37fcccabe2a9</x:v>
+        <x:v>14d064d694dc478f36bb570e78e29368a0259693dfb7217c05975c508bd01db8</x:v>
       </x:c>
       <x:c r="F62" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5067,15 +5272,15 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="97" t="str">
-        <x:v>RECORD-1910_frederick-carrie-doris-andrew-marsh_us-census</x:v>
+        <x:v>RECORD-1901_mayflower-descendant-vol3_john-doane-will</x:v>
       </x:c>
       <x:c r="B63" s="97" t="str">
-        <x:v>1910_frederick-carrie-doris-andrew-marsh_us-census.jpg</x:v>
+        <x:v>1901_mayflower-descendant-vol3_john-doane-will.pdf</x:v>
       </x:c>
       <x:c r="C63" s="97" t="str"/>
       <x:c r="D63" s="97" t="str"/>
       <x:c r="E63" s="97" t="str">
-        <x:v>88afa43f7bb90fc8248f9158ccae50b081e820e9e690022c2ec446434ce47bf4</x:v>
+        <x:v>4d7d359130d69d3db9e5ebdec3f22833c097c0e9dad4e5602047f370bd057518</x:v>
       </x:c>
       <x:c r="F63" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5083,15 +5288,15 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="97" t="str">
-        <x:v>RECORD-1910_henry-madie-charles-vollmer_us-census</x:v>
+        <x:v>RECORD-1904_mayflower-descendant-vol6_eastham-vital-records</x:v>
       </x:c>
       <x:c r="B64" s="97" t="str">
-        <x:v>1910_henry-madie-charles-vollmer_us-census.jpg</x:v>
+        <x:v>1904_mayflower-descendant-vol6_eastham-vital-records.pdf</x:v>
       </x:c>
       <x:c r="C64" s="97" t="str"/>
       <x:c r="D64" s="97" t="str"/>
       <x:c r="E64" s="97" t="str">
-        <x:v>5506a666f811c403bc06da8594751a45791c6f2f60ec7d61bf02be7d70f5bade</x:v>
+        <x:v>105a13412229bb5489c9e245faa82209405ec7199e5fe371dc17a09d1351ba3a</x:v>
       </x:c>
       <x:c r="F64" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5099,15 +5304,15 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="97" t="str">
-        <x:v>RECORD-1917-03-10_frederick-g-vollmer_death-certificate</x:v>
+        <x:v>RECORD-1905-08-05_henry-jj-vollmer_marriage-certificate</x:v>
       </x:c>
       <x:c r="B65" s="97" t="str">
-        <x:v>1917-03-10_frederick-g-vollmer_death-certificate.pdf</x:v>
+        <x:v>1905-08-05_henry-jj-vollmer_marriage-certificate.pdf</x:v>
       </x:c>
       <x:c r="C65" s="97" t="str"/>
       <x:c r="D65" s="97" t="str"/>
       <x:c r="E65" s="97" t="str">
-        <x:v>eb970b4f9f3954c566fe8b3cd5d245162172d247dfc39f93aec396307c88bfc1</x:v>
+        <x:v>59b537c81462fcba56c9827e5a015dacefafd451442735b8db6a37fcccabe2a9</x:v>
       </x:c>
       <x:c r="F65" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5115,15 +5320,15 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="97" t="str">
-        <x:v>RECORD-1918_henry-john-joseph-volmer_wwi-draft-card</x:v>
+        <x:v>RECORD-1910_frederick-carrie-doris-andrew-marsh_us-census</x:v>
       </x:c>
       <x:c r="B66" s="97" t="str">
-        <x:v>1918_henry-john-joseph-volmer_wwi-draft-card.jpg</x:v>
+        <x:v>1910_frederick-carrie-doris-andrew-marsh_us-census.jpg</x:v>
       </x:c>
       <x:c r="C66" s="97" t="str"/>
       <x:c r="D66" s="97" t="str"/>
       <x:c r="E66" s="97" t="str">
-        <x:v>6a929ffb761b504b27bc2cdf2f905fc2ea0b7351cd0554fdd8f38256494367f6</x:v>
+        <x:v>88afa43f7bb90fc8248f9158ccae50b081e820e9e690022c2ec446434ce47bf4</x:v>
       </x:c>
       <x:c r="F66" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5131,15 +5336,15 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="97" t="str">
-        <x:v>RECORD-1919-01-03_madie-vollmer_death-certificate</x:v>
+        <x:v>RECORD-1910_henry-madie-charles-vollmer_us-census</x:v>
       </x:c>
       <x:c r="B67" s="97" t="str">
-        <x:v>1919-01-03_madie-vollmer_death-certificate.pdf</x:v>
+        <x:v>1910_henry-madie-charles-vollmer_us-census.jpg</x:v>
       </x:c>
       <x:c r="C67" s="97" t="str"/>
       <x:c r="D67" s="97" t="str"/>
       <x:c r="E67" s="97" t="str">
-        <x:v>8f8be8c3cb340d5032a2d61e4ed5b578e782c0176054592aee8e48abe1174734</x:v>
+        <x:v>5506a666f811c403bc06da8594751a45791c6f2f60ec7d61bf02be7d70f5bade</x:v>
       </x:c>
       <x:c r="F67" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5147,15 +5352,15 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="97" t="str">
-        <x:v>RECORD-1919-12-17_mary-mcnaughton_ny-death-index</x:v>
+        <x:v>RECORD-1917-03-10_frederick-g-vollmer_death-certificate</x:v>
       </x:c>
       <x:c r="B68" s="97" t="str">
-        <x:v>1919-12-17_mary-mcnaughton_ny-death-index.jpg</x:v>
+        <x:v>1917-03-10_frederick-g-vollmer_death-certificate.pdf</x:v>
       </x:c>
       <x:c r="C68" s="97" t="str"/>
       <x:c r="D68" s="97" t="str"/>
       <x:c r="E68" s="97" t="str">
-        <x:v>2ccad7fd75e95b52575500ee7ff48c3285db4b0d6680654727bf58c704044b3d</x:v>
+        <x:v>eb970b4f9f3954c566fe8b3cd5d245162172d247dfc39f93aec396307c88bfc1</x:v>
       </x:c>
       <x:c r="F68" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5163,15 +5368,15 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="97" t="str">
-        <x:v>RECORD-1940-10-16_charles-frederick-vollmer_wwii-draft-card</x:v>
+        <x:v>RECORD-1918_henry-john-joseph-volmer_wwi-draft-card</x:v>
       </x:c>
       <x:c r="B69" s="97" t="str">
-        <x:v>1940-10-16_charles-frederick-vollmer_wwii-draft-card.jpg</x:v>
+        <x:v>1918_henry-john-joseph-volmer_wwi-draft-card.jpg</x:v>
       </x:c>
       <x:c r="C69" s="97" t="str"/>
       <x:c r="D69" s="97" t="str"/>
       <x:c r="E69" s="97" t="str">
-        <x:v>e755e1f176b897bc6ea96a2ad3bf6697b9634d65f315c438ebefa97638897160</x:v>
+        <x:v>6a929ffb761b504b27bc2cdf2f905fc2ea0b7351cd0554fdd8f38256494367f6</x:v>
       </x:c>
       <x:c r="F69" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5179,15 +5384,15 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="97" t="str">
-        <x:v>RECORD-1940_charles-doris-henry-vollmer_us-census</x:v>
+        <x:v>RECORD-1919-01-03_madie-vollmer_death-certificate</x:v>
       </x:c>
       <x:c r="B70" s="97" t="str">
-        <x:v>1940_charles-doris-henry-vollmer_us-census.jpg</x:v>
+        <x:v>1919-01-03_madie-vollmer_death-certificate.pdf</x:v>
       </x:c>
       <x:c r="C70" s="97" t="str"/>
       <x:c r="D70" s="97" t="str"/>
       <x:c r="E70" s="97" t="str">
-        <x:v>408d8f6dd3a769e32af16d8cc59f762113000942a482dafa1b9ea01431c71ebb</x:v>
+        <x:v>8f8be8c3cb340d5032a2d61e4ed5b578e782c0176054592aee8e48abe1174734</x:v>
       </x:c>
       <x:c r="F70" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5195,15 +5400,15 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="97" t="str">
-        <x:v>RECORD-giles-hopkins_17th-century-records_pilgrim-hall</x:v>
+        <x:v>RECORD-1919-12-17_mary-mcnaughton_ny-death-index</x:v>
       </x:c>
       <x:c r="B71" s="97" t="str">
-        <x:v>giles-hopkins_17th-century-records_pilgrim-hall.pdf</x:v>
+        <x:v>1919-12-17_mary-mcnaughton_ny-death-index.jpg</x:v>
       </x:c>
       <x:c r="C71" s="97" t="str"/>
       <x:c r="D71" s="97" t="str"/>
       <x:c r="E71" s="97" t="str">
-        <x:v>1dbca70bd43b7dd62a3e12bc3b9ee230d8baa0dd37b80cc53ab48ec757763e01</x:v>
+        <x:v>2ccad7fd75e95b52575500ee7ff48c3285db4b0d6680654727bf58c704044b3d</x:v>
       </x:c>
       <x:c r="F71" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5211,15 +5416,15 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="97" t="str">
-        <x:v>RECORD-plymouth-colony-records-vol1_1639-marriage</x:v>
+        <x:v>RECORD-1940-10-16_charles-frederick-vollmer_wwii-draft-card</x:v>
       </x:c>
       <x:c r="B72" s="97" t="str">
-        <x:v>plymouth-colony-records-vol1_1639-marriage.pdf</x:v>
+        <x:v>1940-10-16_charles-frederick-vollmer_wwii-draft-card.jpg</x:v>
       </x:c>
       <x:c r="C72" s="97" t="str"/>
       <x:c r="D72" s="97" t="str"/>
       <x:c r="E72" s="97" t="str">
-        <x:v>243bba40de735bf7deedf4046c40f190526cb1c5cc891ef97a348248067d6cbd</x:v>
+        <x:v>e755e1f176b897bc6ea96a2ad3bf6697b9634d65f315c438ebefa97638897160</x:v>
       </x:c>
       <x:c r="F72" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5227,24 +5432,88 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="97" t="str">
-        <x:v>RECORD-relief-mcnaughton_mother-pension-index</x:v>
+        <x:v>RECORD-1940_charles-doris-henry-vollmer_us-census</x:v>
       </x:c>
       <x:c r="B73" s="97" t="str">
-        <x:v>relief-mcnaughton_mother-pension-index.jpg</x:v>
+        <x:v>1940_charles-doris-henry-vollmer_us-census.jpg</x:v>
       </x:c>
       <x:c r="C73" s="97" t="str"/>
       <x:c r="D73" s="97" t="str"/>
       <x:c r="E73" s="97" t="str">
+        <x:v>408d8f6dd3a769e32af16d8cc59f762113000942a482dafa1b9ea01431c71ebb</x:v>
+      </x:c>
+      <x:c r="F73" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="97" t="str">
+        <x:v>RECORD-1950_william-alice-mary-thoren_us-census</x:v>
+      </x:c>
+      <x:c r="B74" s="97" t="str">
+        <x:v>1950_william-alice-mary-thoren_us-census.jpg</x:v>
+      </x:c>
+      <x:c r="C74" s="97" t="str"/>
+      <x:c r="D74" s="97" t="str"/>
+      <x:c r="E74" s="97" t="str">
+        <x:v>f7e7dde0bcc80447fef0ed66c9699bf2477115f8ea97a2d464724c28c4bb7db5</x:v>
+      </x:c>
+      <x:c r="F74" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="97" t="str">
+        <x:v>RECORD-giles-hopkins_17th-century-records_pilgrim-hall</x:v>
+      </x:c>
+      <x:c r="B75" s="97" t="str">
+        <x:v>giles-hopkins_17th-century-records_pilgrim-hall.pdf</x:v>
+      </x:c>
+      <x:c r="C75" s="97" t="str"/>
+      <x:c r="D75" s="97" t="str"/>
+      <x:c r="E75" s="97" t="str">
+        <x:v>1dbca70bd43b7dd62a3e12bc3b9ee230d8baa0dd37b80cc53ab48ec757763e01</x:v>
+      </x:c>
+      <x:c r="F75" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="97" t="str">
+        <x:v>RECORD-plymouth-colony-records-vol1_1639-marriage</x:v>
+      </x:c>
+      <x:c r="B76" s="97" t="str">
+        <x:v>plymouth-colony-records-vol1_1639-marriage.pdf</x:v>
+      </x:c>
+      <x:c r="C76" s="97" t="str"/>
+      <x:c r="D76" s="97" t="str"/>
+      <x:c r="E76" s="97" t="str">
+        <x:v>243bba40de735bf7deedf4046c40f190526cb1c5cc891ef97a348248067d6cbd</x:v>
+      </x:c>
+      <x:c r="F76" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="97" t="str">
+        <x:v>RECORD-relief-mcnaughton_mother-pension-index</x:v>
+      </x:c>
+      <x:c r="B77" s="97" t="str">
+        <x:v>relief-mcnaughton_mother-pension-index.jpg</x:v>
+      </x:c>
+      <x:c r="C77" s="97" t="str"/>
+      <x:c r="D77" s="97" t="str"/>
+      <x:c r="E77" s="97" t="str">
         <x:v>4c481d5447084325803d01ea3fb19e1485b4d96fd24cc06c3c83ed32580e90f7</x:v>
       </x:c>
-      <x:c r="F73" s="97" t="str">
+      <x:c r="F77" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3fdbc4ba24a4d46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05c0ab30a9a04cac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5312,15 +5581,15 @@
         <x:v>Individuals</x:v>
       </x:c>
       <x:c r="B5" s="92" t="n">
-        <x:f>COUNTA('Consolidated People'!$A$2:$A$309)</x:f>
-        <x:v>308</x:v>
+        <x:f>COUNTA('Consolidated People'!$A$2:$A$311)</x:f>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="C5" s="80"/>
       <x:c r="D5" s="94" t="str">
         <x:v>Jan is Fredric's biological mother</x:v>
       </x:c>
       <x:c r="E5" s="95" t="str">
-        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$309,"Jan Muller Vollmer")=1,"Confirmed","Review")</x:f>
+        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$311,"Jan Muller Vollmer")=1,"Confirmed","Review")</x:f>
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
@@ -5332,19 +5601,19 @@
         <x:v>Families</x:v>
       </x:c>
       <x:c r="B6" s="92" t="n">
-        <x:f>COUNTA('Consolidated Families'!$A$2:$A$145)</x:f>
-        <x:v>144</x:v>
+        <x:f>COUNTA('Consolidated Families'!$A$2:$A$147)</x:f>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="C6" s="80"/>
       <x:c r="D6" s="94" t="str">
-        <x:v>Mary Alice is Chris Vollmer's mother</x:v>
+        <x:v>Mary Alice Thoren identity and parents</x:v>
       </x:c>
       <x:c r="E6" s="95" t="str">
-        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$309,"Mary Alice")=1,"Confirmed","Review")</x:f>
+        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$311,"Mary Alice Thoren")=1,"Confirmed","Review")</x:f>
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="F6" s="94" t="str">
-        <x:v>Biological parent link retained for Chris</x:v>
+        <x:v>Port Townsend birthplace; William J. Thoren and Alice Gallaher parent links; first marriage to Henry recorded</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -5352,8 +5621,8 @@
         <x:v>GEDCOM source records</x:v>
       </x:c>
       <x:c r="B7" s="92" t="n">
-        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$31)</x:f>
-        <x:v>30</x:v>
+        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$34)</x:f>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C7" s="80"/>
       <x:c r="D7" s="94" t="str">
@@ -5371,8 +5640,8 @@
         <x:v>Source and record inventory items</x:v>
       </x:c>
       <x:c r="B8" s="92" t="n">
-        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$73)</x:f>
-        <x:v>72</x:v>
+        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$77)</x:f>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C8" s="80"/>
       <x:c r="D8" s="94" t="str">
@@ -5435,7 +5704,7 @@
         <x:v>Canonical tree structure</x:v>
       </x:c>
       <x:c r="C12" s="97" t="n">
-        <x:v>308</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="D12" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree.ged</x:v>
@@ -5455,7 +5724,7 @@
         <x:v>Structured mirror</x:v>
       </x:c>
       <x:c r="C13" s="97" t="n">
-        <x:v>308</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="D13" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_Canonical_Data.json</x:v>
@@ -5475,7 +5744,7 @@
         <x:v>Person-level audit</x:v>
       </x:c>
       <x:c r="C14" s="97" t="n">
-        <x:v>308</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="D14" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_People.csv</x:v>
@@ -5495,7 +5764,7 @@
         <x:v>Family-level audit</x:v>
       </x:c>
       <x:c r="C15" s="97" t="n">
-        <x:v>144</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D15" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_Families.csv</x:v>
@@ -5504,7 +5773,7 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="F15" s="97" t="str">
-        <x:v>Parent, spouse, and child links</x:v>
+        <x:v>Parent, spouse, child, and marriage links</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
@@ -5515,7 +5784,7 @@
         <x:v>Citation and record index</x:v>
       </x:c>
       <x:c r="C16" s="97" t="n">
-        <x:v>72</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D16" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_Source_Inventory.csv</x:v>
@@ -5524,7 +5793,7 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="F16" s="97" t="str">
-        <x:v>Includes 30 GEDCOM sources and 42 preserved record files</x:v>
+        <x:v>Includes 33 GEDCOM sources and 43 preserved record files</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
@@ -17350,7 +17619,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50aa5daa162d4221"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba13ba4ee81244b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21477,7 +21746,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8ab1230449c4aef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45801b7cd50d4430"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24406,7 +24675,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d563b8085d04a28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6414ae9a140140f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24760,7 +25029,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R007b493cf1594025"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7753d20305974470"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24954,7 +25223,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb8617a96a2148f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4061f468d13b4f5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25432,7 +25701,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rced9314e320846e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fb2a23c99824333"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26515,7 +26784,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1d8b07f49fa4f1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd7ae87e44564e7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31298,16 +31567,16 @@
         <x:v>EXISTING-HENRY-RICHARD-VOLLMER</x:v>
       </x:c>
       <x:c r="G172" s="97" t="str">
-        <x:v>S28</x:v>
+        <x:v>S28;S31</x:v>
       </x:c>
       <x:c r="H172" s="97" t="str">
-        <x:v>Relationship to Fredric: Father. | Confidence: A - Confirmed. | Henry is Fredric's father and Jan's spouse in this tree.</x:v>
+        <x:v>Relationship to Fredric: Father. | Confidence: A - Confirmed. | Henry is Fredric's father and Jan's spouse in this tree. | Owner-confirmed: Mary Alice Thoren was Henry's first wife, before Jan Muller Vollmer.</x:v>
       </x:c>
       <x:c r="I172" s="97" t="str">
         <x:v>F105</x:v>
       </x:c>
       <x:c r="J172" s="97" t="str">
-        <x:v>F095</x:v>
+        <x:v>F095;F146</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -35175,25 +35444,29 @@
         <x:v>I334</x:v>
       </x:c>
       <x:c r="B308" s="97" t="str">
-        <x:v>Mary Alice</x:v>
+        <x:v>Mary Alice Thoren</x:v>
       </x:c>
       <x:c r="C308" s="97" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="D308" s="97" t="str"/>
+      <x:c r="D308" s="97" t="str">
+        <x:v>Port Townsend, Jefferson, Washington</x:v>
+      </x:c>
       <x:c r="E308" s="97" t="str"/>
       <x:c r="F308" s="97" t="str">
         <x:v>OWNER-MARY-ALICE</x:v>
       </x:c>
       <x:c r="G308" s="97" t="str">
-        <x:v>S28</x:v>
+        <x:v>S28;S31;S32</x:v>
       </x:c>
       <x:c r="H308" s="97" t="str">
-        <x:v>Owner-confirmed biological mother of Chris Vollmer. No surname or other living details inferred.</x:v>
-      </x:c>
-      <x:c r="I308" s="97" t="str"/>
+        <x:v>Owner-confirmed biological mother of Chris Vollmer and first wife of Henry Richard Vollmer, before Jan Muller Vollmer. | Owner-confirmed birthplace: Port Townsend, Washington. Exact birth date omitted for privacy. | The 1950 census identifies her as the daughter of William J. Thoren and Alice Gallaher Thoren. | Potentially living; details are minimized.</x:v>
+      </x:c>
+      <x:c r="I308" s="97" t="str">
+        <x:v>F145</x:v>
+      </x:c>
       <x:c r="J308" s="97" t="str">
-        <x:v>F144</x:v>
+        <x:v>F144;F146</x:v>
       </x:c>
     </x:row>
     <x:row r="309">
@@ -35222,10 +35495,66 @@
       </x:c>
       <x:c r="J309" s="97" t="str"/>
     </x:row>
+    <x:row r="310">
+      <x:c r="A310" s="97" t="str">
+        <x:v>I336</x:v>
+      </x:c>
+      <x:c r="B310" s="97" t="str">
+        <x:v>William J Thoren</x:v>
+      </x:c>
+      <x:c r="C310" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D310" s="97" t="str">
+        <x:v>ABT 1902; Montana</x:v>
+      </x:c>
+      <x:c r="E310" s="97" t="str"/>
+      <x:c r="F310" s="97" t="str">
+        <x:v>OWNER-WILLIAM-J-THOREN</x:v>
+      </x:c>
+      <x:c r="G310" s="97" t="str">
+        <x:v>S28;S32;S33</x:v>
+      </x:c>
+      <x:c r="H310" s="97" t="str">
+        <x:v>Called Bill in family memory. The 1950 census records him as age 48, born in Montana, and Mary Alice's father.</x:v>
+      </x:c>
+      <x:c r="I310" s="97" t="str"/>
+      <x:c r="J310" s="97" t="str">
+        <x:v>F145</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="311">
+      <x:c r="A311" s="97" t="str">
+        <x:v>I337</x:v>
+      </x:c>
+      <x:c r="B311" s="97" t="str">
+        <x:v>Alice Gallaher</x:v>
+      </x:c>
+      <x:c r="C311" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D311" s="97" t="str">
+        <x:v>ABT 1904; Alaska</x:v>
+      </x:c>
+      <x:c r="E311" s="97" t="str"/>
+      <x:c r="F311" s="97" t="str">
+        <x:v>RECORD-ALICE-GALLAHER-THOREN</x:v>
+      </x:c>
+      <x:c r="G311" s="97" t="str">
+        <x:v>S32;S33</x:v>
+      </x:c>
+      <x:c r="H311" s="97" t="str">
+        <x:v>The 1950 census records her as age 46, born in Alaska, and Mary Alice's mother; her 1929 marriage record supplies the maiden surname Gallaher.</x:v>
+      </x:c>
+      <x:c r="I311" s="97" t="str"/>
+      <x:c r="J311" s="97" t="str">
+        <x:v>F145</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R075838eae354468e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761ebfc8d3ed4ab2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Confirm Henry as Chris's father
</commit_message>
<xml_diff>
--- a/original-data/final-family-tree/Fredric_Vollmer_Complete_Family_Tree_Index.xlsx
+++ b/original-data/final-family-tree/Fredric_Vollmer_Complete_Family_Tree_Index.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rd876436d6c344821"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancestor Index" sheetId="2" r:id="Raedecbfabe5244df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="3" r:id="R9724e9810991473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended Family" sheetId="4" r:id="Rbd782cfff06848ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household Audit" sheetId="5" r:id="R35014b64b8884ed6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correction Log" sheetId="6" r:id="R079ee3222f5b48c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Gaps" sheetId="7" r:id="Re8853001e90f4d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Key" sheetId="8" r:id="R0aad920191204719"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated People" sheetId="9" r:id="Rbdf6ed21aad04bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Families" sheetId="10" r:id="Ra891baee4ff74c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Sources" sheetId="11" r:id="Rc62711123b0943d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Overview" sheetId="12" r:id="R73a3aaa9ebd34d98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R6f5e60e1beaa4819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancestor Index" sheetId="2" r:id="Rc67ddecc64df470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="3" r:id="R4b184eebb2d44245"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended Family" sheetId="4" r:id="R8be841bd88cb465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household Audit" sheetId="5" r:id="Rfe002044a02f44f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correction Log" sheetId="6" r:id="Rd131c16a834a4e12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Gaps" sheetId="7" r:id="R4f75443f44a542a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Key" sheetId="8" r:id="Re171fdfd53b14638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated People" sheetId="9" r:id="Rd3b3f8484be64bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Families" sheetId="10" r:id="R7f23a211944c4430"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Sources" sheetId="11" r:id="Redd2fc15105a4c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Overview" sheetId="12" r:id="R97e8a4bf43c6432d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -678,7 +678,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5fd8d5d2a1e94dae"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R22d8b8e0f5b34956"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -844,8 +844,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ConsolidatedFamiliesTable" displayName="ConsolidatedFamiliesTable" ref="A1:G147" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:G147"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ConsolidatedFamiliesTable" displayName="ConsolidatedFamiliesTable" ref="A1:G146" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G146"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="family_id"/>
     <x:tableColumn id="2" name="husband_id"/>
@@ -1534,7 +1534,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R802a8f5369b74a0e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a188147f9c740fb"/>
 </x:worksheet>
 </file>
 
@@ -4167,19 +4167,23 @@
       <x:c r="A145" s="97" t="str">
         <x:v>F144</x:v>
       </x:c>
-      <x:c r="B145" s="97" t="str"/>
+      <x:c r="B145" s="97" t="str">
+        <x:v>I176</x:v>
+      </x:c>
       <x:c r="C145" s="97" t="str">
         <x:v>I334</x:v>
       </x:c>
       <x:c r="D145" s="97" t="str">
         <x:v>I335</x:v>
       </x:c>
-      <x:c r="E145" s="97" t="str"/>
+      <x:c r="E145" s="97" t="str">
+        <x:v>16 SEP 1955; King County, Washington</x:v>
+      </x:c>
       <x:c r="F145" s="97" t="str">
-        <x:v>Chris's father was not confirmed and is intentionally omitted.</x:v>
+        <x:v>Owner-confirmed biological parents of Chris Vollmer. Chris is Fredric Muller Vollmer's paternal half-brother. The earlier unconfirmed-father status is superseded by the owner's 2 September 2026 clarification. | Washington State Archives documents Henry and Mary Alice's marriage; owner testimony separately confirms both as Chris's biological parents.</x:v>
       </x:c>
       <x:c r="G145" s="97" t="str">
-        <x:v>S28</x:v>
+        <x:v>S28;S31</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -4205,31 +4209,10 @@
         <x:v>S32;S33</x:v>
       </x:c>
     </x:row>
-    <x:row r="147">
-      <x:c r="A147" s="97" t="str">
-        <x:v>F146</x:v>
-      </x:c>
-      <x:c r="B147" s="97" t="str">
-        <x:v>I176</x:v>
-      </x:c>
-      <x:c r="C147" s="97" t="str">
-        <x:v>I334</x:v>
-      </x:c>
-      <x:c r="D147" s="97" t="str"/>
-      <x:c r="E147" s="97" t="str">
-        <x:v>16 SEP 1955; King County, Washington</x:v>
-      </x:c>
-      <x:c r="F147" s="97" t="str">
-        <x:v>Owner-confirmed first marriage of Henry, before his marriage to Jan. This spouse link does not establish Chris's father.</x:v>
-      </x:c>
-      <x:c r="G147" s="97" t="str">
-        <x:v>S28;S31</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42c39c52c2cb4e0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R450798debbd249f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4716,7 +4699,7 @@
         <x:v>2 SEP 2026</x:v>
       </x:c>
       <x:c r="E29" s="97" t="str">
-        <x:v>Jan is Fredric's biological mother; Mary Alice Thoren was born in Port Townsend, was Henry's first wife, and is Chris Vollmer's mother; Jan is Chris's stepmother. William 'Bill' Thoren was remembered as Mary Alice's father. Chris's father was not stated.</x:v>
+        <x:v>Jan is Fredric's biological mother; Mary Alice Thoren was born in Port Townsend, was Henry's first wife, and is Chris Vollmer's mother; Jan is Chris's stepmother. William 'Bill' Thoren was remembered as Mary Alice's father. A later 2 Sep statement explicitly identifies Henry as Chris's biological father and Chris as Fredric's paternal half-brother, superseding the earlier unconfirmed status.</x:v>
       </x:c>
       <x:c r="F29" s="97" t="str">
         <x:v>cross-chat consolidation</x:v>
@@ -5513,7 +5496,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05c0ab30a9a04cac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R029ba46886db4a0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5601,8 +5584,8 @@
         <x:v>Families</x:v>
       </x:c>
       <x:c r="B6" s="92" t="n">
-        <x:f>COUNTA('Consolidated Families'!$A$2:$A$147)</x:f>
-        <x:v>146</x:v>
+        <x:f>COUNTA('Consolidated Families'!$A$2:$A$146)</x:f>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="C6" s="80"/>
       <x:c r="D6" s="94" t="str">
@@ -5647,11 +5630,11 @@
       <x:c r="D8" s="94" t="str">
         <x:v>Chris's father</x:v>
       </x:c>
-      <x:c r="E8" s="94" t="str">
-        <x:v>Intentionally blank</x:v>
+      <x:c r="E8" s="95" t="str">
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="F8" s="94" t="str">
-        <x:v>Not inferred from available evidence</x:v>
+        <x:v>Henry and Mary Alice are the biological parents; Chris is Fredric's paternal half-brother</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -5764,7 +5747,7 @@
         <x:v>Family-level audit</x:v>
       </x:c>
       <x:c r="C15" s="97" t="n">
-        <x:v>146</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D15" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_Families.csv</x:v>
@@ -17619,7 +17602,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba13ba4ee81244b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95657ae8b9b34f09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21746,7 +21729,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45801b7cd50d4430"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f66bbbe0868449e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24675,7 +24658,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6414ae9a140140f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb61ca122ff65431b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25029,7 +25012,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7753d20305974470"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23624991a5784c13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25223,7 +25206,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4061f468d13b4f5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48e9016022654a7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25701,7 +25684,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fb2a23c99824333"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re747d8b77caf4964"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26784,7 +26767,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd7ae87e44564e7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41c4f7e1ecbc4482"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31570,13 +31553,13 @@
         <x:v>S28;S31</x:v>
       </x:c>
       <x:c r="H172" s="97" t="str">
-        <x:v>Relationship to Fredric: Father. | Confidence: A - Confirmed. | Henry is Fredric's father and Jan's spouse in this tree. | Owner-confirmed: Mary Alice Thoren was Henry's first wife, before Jan Muller Vollmer.</x:v>
+        <x:v>Relationship to Fredric: Father. | Confidence: A - Confirmed. | Henry is Fredric's father and Jan's spouse in this tree. | Owner-confirmed: Mary Alice Thoren was Henry's first wife, before Jan Muller Vollmer. | Owner-confirmed: Henry is Chris Vollmer's biological father; Chris is Fredric's paternal half-brother.</x:v>
       </x:c>
       <x:c r="I172" s="97" t="str">
         <x:v>F105</x:v>
       </x:c>
       <x:c r="J172" s="97" t="str">
-        <x:v>F095;F146</x:v>
+        <x:v>F095;F144</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -35460,13 +35443,13 @@
         <x:v>S28;S31;S32</x:v>
       </x:c>
       <x:c r="H308" s="97" t="str">
-        <x:v>Owner-confirmed biological mother of Chris Vollmer and first wife of Henry Richard Vollmer, before Jan Muller Vollmer. | Owner-confirmed birthplace: Port Townsend, Washington. Exact birth date omitted for privacy. | The 1950 census identifies her as the daughter of William J. Thoren and Alice Gallaher Thoren. | Potentially living; details are minimized.</x:v>
+        <x:v>Owner-confirmed biological mother of Chris Vollmer and first wife of Henry Richard Vollmer, before Jan Muller Vollmer. Henry and Mary Alice are Chris's biological parents. | Owner-confirmed birthplace: Port Townsend, Washington. Exact birth date omitted for privacy. | The 1950 census identifies her as the daughter of William J. Thoren and Alice Gallaher Thoren. | Potentially living; details are minimized.</x:v>
       </x:c>
       <x:c r="I308" s="97" t="str">
         <x:v>F145</x:v>
       </x:c>
       <x:c r="J308" s="97" t="str">
-        <x:v>F144;F146</x:v>
+        <x:v>F144</x:v>
       </x:c>
     </x:row>
     <x:row r="309">
@@ -35488,7 +35471,7 @@
         <x:v>S28</x:v>
       </x:c>
       <x:c r="H309" s="97" t="str">
-        <x:v>Owner-confirmed child of Mary Alice and stepchild of Jan Muller Vollmer. Father not confirmed and intentionally left blank.</x:v>
+        <x:v>Owner-confirmed son of Henry Richard Vollmer and Mary Alice Thoren, stepchild of Jan Muller Vollmer, and paternal half-brother of Fredric Muller Vollmer.</x:v>
       </x:c>
       <x:c r="I309" s="97" t="str">
         <x:v>F144</x:v>
@@ -35554,7 +35537,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761ebfc8d3ed4ab2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b7c03ac683240ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Extend Mary Alice Thoren ancestry into Sweden
</commit_message>
<xml_diff>
--- a/original-data/final-family-tree/Fredric_Vollmer_Complete_Family_Tree_Index.xlsx
+++ b/original-data/final-family-tree/Fredric_Vollmer_Complete_Family_Tree_Index.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R6f5e60e1beaa4819"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancestor Index" sheetId="2" r:id="Rc67ddecc64df470e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="3" r:id="R4b184eebb2d44245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended Family" sheetId="4" r:id="R8be841bd88cb465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household Audit" sheetId="5" r:id="Rfe002044a02f44f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correction Log" sheetId="6" r:id="Rd131c16a834a4e12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Gaps" sheetId="7" r:id="R4f75443f44a542a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Key" sheetId="8" r:id="Re171fdfd53b14638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated People" sheetId="9" r:id="Rd3b3f8484be64bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Families" sheetId="10" r:id="R7f23a211944c4430"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Sources" sheetId="11" r:id="Redd2fc15105a4c66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Overview" sheetId="12" r:id="R97e8a4bf43c6432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R7998e1d97cd24354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancestor Index" sheetId="2" r:id="R48bcd30ae6fe4dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="3" r:id="Ra8fcff4fc86240e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended Family" sheetId="4" r:id="R455cdc5ba89b4260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household Audit" sheetId="5" r:id="R60d49faf6bd54008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correction Log" sheetId="6" r:id="R909bfea19f414706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Gaps" sheetId="7" r:id="R55044822add940bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Key" sheetId="8" r:id="Rdf7500cc9da042ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated People" sheetId="9" r:id="R7242d0182cbe4433"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Families" sheetId="10" r:id="R2b35fb6be1ee42c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Sources" sheetId="11" r:id="Rc3535147646f424f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Overview" sheetId="12" r:id="R6bbbf5997497424f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -678,7 +678,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R22d8b8e0f5b34956"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9831cbd983fe4348"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -714,8 +714,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ConsolidatedSourcesTable" displayName="ConsolidatedSourcesTable" ref="A1:F77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F77"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ConsolidatedSourcesTable" displayName="ConsolidatedSourcesTable" ref="A1:F89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F89"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="source_id"/>
     <x:tableColumn id="2" name="title"/>
@@ -825,8 +825,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ConsolidatedPeopleTable" displayName="ConsolidatedPeopleTable" ref="A1:J311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J311"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ConsolidatedPeopleTable" displayName="ConsolidatedPeopleTable" ref="A1:J328" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J328"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="individual_id"/>
     <x:tableColumn id="2" name="name"/>
@@ -844,8 +844,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ConsolidatedFamiliesTable" displayName="ConsolidatedFamiliesTable" ref="A1:G146" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:G146"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ConsolidatedFamiliesTable" displayName="ConsolidatedFamiliesTable" ref="A1:G155" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G155"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="family_id"/>
     <x:tableColumn id="2" name="husband_id"/>
@@ -1534,7 +1534,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a188147f9c740fb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R518f3c7d1b2b47ba"/>
 </x:worksheet>
 </file>
 
@@ -4209,10 +4209,199 @@
         <x:v>S32;S33</x:v>
       </x:c>
     </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="97" t="str">
+        <x:v>F146</x:v>
+      </x:c>
+      <x:c r="B147" s="97" t="str">
+        <x:v>I338</x:v>
+      </x:c>
+      <x:c r="C147" s="97" t="str">
+        <x:v>I339</x:v>
+      </x:c>
+      <x:c r="D147" s="97" t="str">
+        <x:v>I336</x:v>
+      </x:c>
+      <x:c r="E147" s="97" t="str"/>
+      <x:c r="F147" s="97" t="str">
+        <x:v>The 1910 Great Falls census records William as the son of Christian and Augusta Thoren; Swedish records identify both parents' earlier generations.</x:v>
+      </x:c>
+      <x:c r="G147" s="97" t="str">
+        <x:v>S34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="97" t="str">
+        <x:v>F147</x:v>
+      </x:c>
+      <x:c r="B148" s="97" t="str">
+        <x:v>I340</x:v>
+      </x:c>
+      <x:c r="C148" s="97" t="str">
+        <x:v>I341</x:v>
+      </x:c>
+      <x:c r="D148" s="97" t="str">
+        <x:v>I338</x:v>
+      </x:c>
+      <x:c r="E148" s="97" t="str"/>
+      <x:c r="F148" s="97" t="str">
+        <x:v>Christian's Swedish indexed birth and the linked household surveys identify Anders and Kjersti as his parents.</x:v>
+      </x:c>
+      <x:c r="G148" s="97" t="str">
+        <x:v>S36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="97" t="str">
+        <x:v>F148</x:v>
+      </x:c>
+      <x:c r="B149" s="97" t="str">
+        <x:v>I342</x:v>
+      </x:c>
+      <x:c r="C149" s="97" t="str">
+        <x:v>I343</x:v>
+      </x:c>
+      <x:c r="D149" s="97" t="str">
+        <x:v>I340</x:v>
+      </x:c>
+      <x:c r="E149" s="97" t="str"/>
+      <x:c r="F149" s="97" t="str">
+        <x:v>The Norra Sandby household survey records Anders as the son of Trued Andersson and Bortha Nilsdotter.</x:v>
+      </x:c>
+      <x:c r="G149" s="97" t="str">
+        <x:v>S38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="97" t="str">
+        <x:v>F149</x:v>
+      </x:c>
+      <x:c r="B150" s="97" t="str">
+        <x:v>I344</x:v>
+      </x:c>
+      <x:c r="C150" s="97" t="str">
+        <x:v>I345</x:v>
+      </x:c>
+      <x:c r="D150" s="97" t="str">
+        <x:v>I339</x:v>
+      </x:c>
+      <x:c r="E150" s="97" t="str">
+        <x:v>26 OCT 1850; Ränneslöv, Halland, Sweden</x:v>
+      </x:c>
+      <x:c r="F150" s="97" t="str">
+        <x:v>Augusta's Hjärnarp birth, baptism, and household records identify Nils and Christina as her parents.</x:v>
+      </x:c>
+      <x:c r="G150" s="97" t="str">
+        <x:v>S37;S39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="97" t="str">
+        <x:v>F150</x:v>
+      </x:c>
+      <x:c r="B151" s="97" t="str"/>
+      <x:c r="C151" s="97" t="str">
+        <x:v>I346</x:v>
+      </x:c>
+      <x:c r="D151" s="97" t="str">
+        <x:v>I344</x:v>
+      </x:c>
+      <x:c r="E151" s="97" t="str"/>
+      <x:c r="F151" s="97" t="str">
+        <x:v>Nils's 1825 baptism names Gunnilla Nilsdotter as his mother and names no father; the father remains blank.</x:v>
+      </x:c>
+      <x:c r="G151" s="97" t="str">
+        <x:v>S40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="97" t="str">
+        <x:v>F151</x:v>
+      </x:c>
+      <x:c r="B152" s="97" t="str">
+        <x:v>I347</x:v>
+      </x:c>
+      <x:c r="C152" s="97" t="str">
+        <x:v>I348</x:v>
+      </x:c>
+      <x:c r="D152" s="97" t="str">
+        <x:v>I346</x:v>
+      </x:c>
+      <x:c r="E152" s="97" t="str"/>
+      <x:c r="F152" s="97" t="str">
+        <x:v>Gunnilla's 1796 baptism names Nils Johansson and Elna Nilsdotter as her parents.</x:v>
+      </x:c>
+      <x:c r="G152" s="97" t="str">
+        <x:v>S41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="97" t="str">
+        <x:v>F152</x:v>
+      </x:c>
+      <x:c r="B153" s="97" t="str">
+        <x:v>I349</x:v>
+      </x:c>
+      <x:c r="C153" s="97" t="str">
+        <x:v>I350</x:v>
+      </x:c>
+      <x:c r="D153" s="97" t="str">
+        <x:v>I345</x:v>
+      </x:c>
+      <x:c r="E153" s="97" t="str"/>
+      <x:c r="F153" s="97" t="str">
+        <x:v>Christina's 1823 baptism and the Hasslöv household survey identify Pehr and Ingier as her parents.</x:v>
+      </x:c>
+      <x:c r="G153" s="97" t="str">
+        <x:v>S42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="97" t="str">
+        <x:v>F153</x:v>
+      </x:c>
+      <x:c r="B154" s="97" t="str">
+        <x:v>I351</x:v>
+      </x:c>
+      <x:c r="C154" s="97" t="str">
+        <x:v>I352</x:v>
+      </x:c>
+      <x:c r="D154" s="97" t="str">
+        <x:v>I349</x:v>
+      </x:c>
+      <x:c r="E154" s="97" t="str"/>
+      <x:c r="F154" s="97" t="str">
+        <x:v>Pehr's 1790 Hishult baptism names Erland Pålsson and Bengta Pehrsdotter as his parents.</x:v>
+      </x:c>
+      <x:c r="G154" s="97" t="str">
+        <x:v>S44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="97" t="str">
+        <x:v>F154</x:v>
+      </x:c>
+      <x:c r="B155" s="97" t="str">
+        <x:v>I353</x:v>
+      </x:c>
+      <x:c r="C155" s="97" t="str">
+        <x:v>I354</x:v>
+      </x:c>
+      <x:c r="D155" s="97" t="str">
+        <x:v>I350</x:v>
+      </x:c>
+      <x:c r="E155" s="97" t="str"/>
+      <x:c r="F155" s="97" t="str">
+        <x:v>Ingier's 1794 Hasslöv baptism names Hans Månsson and Maria Hansdotter as her parents.</x:v>
+      </x:c>
+      <x:c r="G155" s="97" t="str">
+        <x:v>S45</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R450798debbd249f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R310f5186ce884c7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4807,207 +4996,241 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="97" t="str">
-        <x:v>RECORD-1648-06-15_deborah-hopkins_birth-register</x:v>
+        <x:v>S34</x:v>
       </x:c>
       <x:c r="B35" s="97" t="str">
-        <x:v>1648-06-15_deborah-hopkins_birth-register.jpg</x:v>
-      </x:c>
-      <x:c r="C35" s="97" t="str"/>
+        <x:v>William John Thoren U.S. census, draft, and death-record cluster</x:v>
+      </x:c>
+      <x:c r="C35" s="97" t="str">
+        <x:v>U.S. Census Bureau; Selective Service System; state and federal vital-record indexes; Ancestry.com</x:v>
+      </x:c>
       <x:c r="D35" s="97" t="str"/>
       <x:c r="E35" s="97" t="str">
-        <x:v>4e6dd607655f9c2b251e3974596d63276178e76761116b370a8b16e0219f3f98</x:v>
+        <x:v>The 1910 Great Falls census places William, born about 1902 in Montana, as son of Christian and Augusta Thoren; later records establish birth 19 Jul 1901 at Great Falls and death 26 Oct 1991. Records: https://www.ancestry.com/search/collections/7884/records/191842032 ; https://www.ancestry.com/search/collections/6061/records/45709575 ; https://www.ancestry.com/search/collections/6224/records/111918347 ; https://www.ancestry.com/search/collections/2238/records/37117805 ; https://www.ancestry.com/search/collections/5254/records/1097942 ; https://www.ancestry.com/search/collections/3693/records/62441333</x:v>
       </x:c>
       <x:c r="F35" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="97" t="str">
-        <x:v>RECORD-1667-02-05_ephraim-doane_mary-knowles_marriage-register</x:v>
+        <x:v>S35</x:v>
       </x:c>
       <x:c r="B36" s="97" t="str">
-        <x:v>1667-02-05_ephraim-doane_mary-knowles_marriage-register.jpg</x:v>
-      </x:c>
-      <x:c r="C36" s="97" t="str"/>
+        <x:v>Alice Gallaher Thoren U.S. census, Social Security, death, and burial-record cluster</x:v>
+      </x:c>
+      <x:c r="C36" s="97" t="str">
+        <x:v>U.S. Census Bureau; Social Security Administration; Washington State; Find a Grave; Ancestry.com</x:v>
+      </x:c>
       <x:c r="D36" s="97" t="str"/>
       <x:c r="E36" s="97" t="str">
-        <x:v>89ae0910e197b39bd902ca52685d144ab55193a340c5e6d3dbeb15a811487faa</x:v>
+        <x:v>Records establish birth 27 Apr 1902 in Alaska and death 23 Aug 1978 at Ocean Park, Washington, while the 1929 marriage supplies Gallaher. No parent-naming primary record was found. Records: https://www.ancestry.com/search/collections/6224/records/111918337 ; https://www.ancestry.com/search/collections/3693/records/62440948 ; https://www.ancestry.com/search/collections/6716/records/895426 ; https://www.ancestry.com/search/collections/60541/records/182552983 ; https://www.ancestry.com/search/collections/60901/records/778054457</x:v>
       </x:c>
       <x:c r="F36" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="97" t="str">
-        <x:v>RECORD-1682-02-04_joshua-cook_birth-register</x:v>
+        <x:v>S36</x:v>
       </x:c>
       <x:c r="B37" s="97" t="str">
-        <x:v>1682-02-04_joshua-cook_birth-register.jpg</x:v>
-      </x:c>
-      <x:c r="C37" s="97" t="str"/>
+        <x:v>Christian Andrew Thoren Swedish birth and household records, U.S. census, and Montana death index</x:v>
+      </x:c>
+      <x:c r="C37" s="97" t="str">
+        <x:v>ArkivDigital; U.S. Census Bureau; Montana Department of Public Health and Human Services; Ancestry.com</x:v>
+      </x:c>
       <x:c r="D37" s="97" t="str"/>
       <x:c r="E37" s="97" t="str">
-        <x:v>726be1a255bf2abe13e2cdc2d149bcddf7dfb1702c466ab4e215d38133e9ea46</x:v>
+        <x:v>Swedish records identify Christian Andersson/Thorén, born 27 Jan 1861 at Ignaberga, as son of Anders Troedsson and Kjersti Månsdotter. The Montana death index records 9 May 1921 but incorrectly places wife Augusta Nelson in the mother field. Records: https://www.ancestry.com/search/collections/2262/records/40805501 ; https://www.ancestry.com/search/collections/9731/records/42221130 ; https://www.ancestry.com/search/collections/7602/records/76515976 ; https://www.ancestry.com/search/collections/6061/records/45709573 ; https://www.ancestry.com/search/collections/5437/records/820390</x:v>
       </x:c>
       <x:c r="F37" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="97" t="str">
-        <x:v>RECORD-1682-04_patience-doane_birth-register</x:v>
+        <x:v>S37</x:v>
       </x:c>
       <x:c r="B38" s="97" t="str">
-        <x:v>1682-04_patience-doane_birth-register.jpg</x:v>
-      </x:c>
-      <x:c r="C38" s="97" t="str"/>
+        <x:v>Augusta Nilsdotter Thoren Swedish birth, baptism, household, U.S. census, and burial records</x:v>
+      </x:c>
+      <x:c r="C38" s="97" t="str">
+        <x:v>ArkivDigital; FamilySearch; U.S. Census Bureau; Find a Grave; Ancestry.com</x:v>
+      </x:c>
       <x:c r="D38" s="97" t="str"/>
       <x:c r="E38" s="97" t="str">
-        <x:v>c754af467f7252cd6952af7bc5948ce2ca5f77fdb7c7e60a6941088448c32e4a</x:v>
+        <x:v>Records identify Augusta, born 30 Nov 1860 at Hjärnarp, as daughter of Nils Svensson and Christina Persdotter; she died 4 Dec 1913 at Great Falls. Name forms include Nilsdotter, Svensson, Nilson, Nelson, and Thoren. Records: https://www.ancestry.com/search/collections/2262/records/41710407 ; https://www.ancestry.com/search/collections/60361/records/255112 ; https://www.ancestry.com/search/collections/9731/records/29521690 ; https://www.ancestry.com/search/collections/7602/records/76515977 ; https://www.ancestry.com/search/collections/60525/records/24177921</x:v>
       </x:c>
       <x:c r="F38" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="97" t="str">
-        <x:v>RECORD-1696_joshua-lane_birth-record</x:v>
+        <x:v>S38</x:v>
       </x:c>
       <x:c r="B39" s="97" t="str">
-        <x:v>1696_joshua-lane_birth-record.jpg</x:v>
-      </x:c>
-      <x:c r="C39" s="97" t="str"/>
+        <x:v>Anders Troedsson and Kjersti Månsdotter Swedish household-survey chain</x:v>
+      </x:c>
+      <x:c r="C39" s="97" t="str">
+        <x:v>ArkivDigital; Ancestry.com</x:v>
+      </x:c>
       <x:c r="D39" s="97" t="str"/>
       <x:c r="E39" s="97" t="str">
-        <x:v>23c17bccf0b93d5ca970ddc6458dc14f264e129c5650c13a9e613dc57e94371e</x:v>
+        <x:v>The Ignaberga household links Anders (born 2 May 1824) and Kjersti (born 31 Oct 1825) to son Christian; the earlier Norra Sandby household links Anders to parents Trued Andersson (born 25 Apr 1792) and Bortha Nilsdotter (born 1783). Records: https://www.ancestry.com/search/collections/9731/records/8673393 ; https://www.ancestry.com/search/collections/9731/records/8673394 ; https://www.ancestry.com/search/collections/9731/records/73561674 ; https://www.ancestry.com/search/collections/9731/records/73561672 ; https://www.ancestry.com/search/collections/9731/records/73561673</x:v>
       </x:c>
       <x:c r="F39" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="97" t="str">
-        <x:v>RECORD-1717_joshua-lane_bathsheba-robie_marriage-record</x:v>
+        <x:v>S39</x:v>
       </x:c>
       <x:c r="B40" s="97" t="str">
-        <x:v>1717_joshua-lane_bathsheba-robie_marriage-record.jpg</x:v>
-      </x:c>
-      <x:c r="C40" s="97" t="str"/>
+        <x:v>Nils Svensson and Christina Persdotter household and marriage records</x:v>
+      </x:c>
+      <x:c r="C40" s="97" t="str">
+        <x:v>ArkivDigital; FamilySearch; Ancestry.com</x:v>
+      </x:c>
       <x:c r="D40" s="97" t="str"/>
       <x:c r="E40" s="97" t="str">
-        <x:v>15e63b00090b98e21bb4ae4d28cc0d2a620bbe75946c63efe681f5b512fb6b9c</x:v>
+        <x:v>The Hjärnarp household records the couple with daughter Augusta and their birthplaces/dates; the marriage index records 26 Oct 1850 at Ränneslöv. Records: https://www.ancestry.com/search/collections/9731/records/29521684 ; https://www.ancestry.com/search/collections/9731/records/29521685 ; https://www.ancestry.com/search/collections/60363/records/338059 ; https://www.ancestry.com/search/collections/60363/records/338058</x:v>
       </x:c>
       <x:c r="F40" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="97" t="str">
-        <x:v>RECORD-1718_samuel-lane_birth-record</x:v>
+        <x:v>S40</x:v>
       </x:c>
       <x:c r="B41" s="97" t="str">
-        <x:v>1718_samuel-lane_birth-record.jpg</x:v>
-      </x:c>
-      <x:c r="C41" s="97" t="str"/>
-      <x:c r="D41" s="97" t="str"/>
+        <x:v>Nils Svensson 1825 Ränneslöv baptism</x:v>
+      </x:c>
+      <x:c r="C41" s="97" t="str">
+        <x:v>FamilySearch; Ancestry.com</x:v>
+      </x:c>
+      <x:c r="D41" s="97" t="str">
+        <x:v>5 MAY 1825</x:v>
+      </x:c>
       <x:c r="E41" s="97" t="str">
-        <x:v>0200f2252b3392cf2fa2ecb3d58b9ddef31b998ce5d76ef552bfab2ee7eda016</x:v>
+        <x:v>Nils was born 3 May and baptized 5 May 1825 at Ränneslöv. The record names Gunnilla Nilsdotter as mother and names no father, so the paternal link remains blank. https://www.ancestry.com/search/collections/60361/records/13922815</x:v>
       </x:c>
       <x:c r="F41" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="97" t="str">
-        <x:v>RECORD-1722_mary-james_birth-record</x:v>
+        <x:v>S41</x:v>
       </x:c>
       <x:c r="B42" s="97" t="str">
-        <x:v>1722_mary-james_birth-record.jpg</x:v>
-      </x:c>
-      <x:c r="C42" s="97" t="str"/>
-      <x:c r="D42" s="97" t="str"/>
+        <x:v>Gunnilla Nilsdotter 1796 Ränneslöv baptism</x:v>
+      </x:c>
+      <x:c r="C42" s="97" t="str">
+        <x:v>FamilySearch; Ancestry.com</x:v>
+      </x:c>
+      <x:c r="D42" s="97" t="str">
+        <x:v>25 SEP 1796</x:v>
+      </x:c>
       <x:c r="E42" s="97" t="str">
-        <x:v>189899f04cbc5dc801896487041938515771118dabdb1af87ed6662a4f6ffcd9</x:v>
+        <x:v>Gunla/Gunnilla was born 20 Sep and baptized 25 Sep 1796 at Ränneslöv, daughter of Nils Johansson and Elna Nilsdotter. https://www.ancestry.com/search/collections/60361/records/22162419</x:v>
       </x:c>
       <x:c r="F42" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="97" t="str">
-        <x:v>RECORD-1741-12-24_samuel-lane_mary-james_marriage</x:v>
+        <x:v>S42</x:v>
       </x:c>
       <x:c r="B43" s="97" t="str">
-        <x:v>1741-12-24_samuel-lane_mary-james_marriage.jpg</x:v>
-      </x:c>
-      <x:c r="C43" s="97" t="str"/>
-      <x:c r="D43" s="97" t="str"/>
+        <x:v>Christina Persdotter 1823 Hasslöv baptism</x:v>
+      </x:c>
+      <x:c r="C43" s="97" t="str">
+        <x:v>FamilySearch; Ancestry.com</x:v>
+      </x:c>
+      <x:c r="D43" s="97" t="str">
+        <x:v>25 JAN 1823</x:v>
+      </x:c>
       <x:c r="E43" s="97" t="str">
-        <x:v>fd6d017aaaa9f3c51bd77b7c6a0a007e08a6b28b3eacd4323314c75ced5f61b4</x:v>
+        <x:v>Stina/Christina was born 24 Jan and baptized 25 Jan 1823 at Hasslöv, daughter of Pehr Erlandsson and Ingier Hansdotter. https://www.ancestry.com/search/collections/60361/records/23764021</x:v>
       </x:c>
       <x:c r="F43" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="97" t="str">
-        <x:v>RECORD-1748-02-09_joshua-lane_nh-birth</x:v>
+        <x:v>S43</x:v>
       </x:c>
       <x:c r="B44" s="97" t="str">
-        <x:v>1748-02-09_joshua-lane_nh-birth.jpg</x:v>
-      </x:c>
-      <x:c r="C44" s="97" t="str"/>
+        <x:v>Pehr Erlandsson and Ingier Hansdotter Hasslöv household survey</x:v>
+      </x:c>
+      <x:c r="C44" s="97" t="str">
+        <x:v>ArkivDigital; Ancestry.com</x:v>
+      </x:c>
       <x:c r="D44" s="97" t="str"/>
       <x:c r="E44" s="97" t="str">
-        <x:v>8b75cc1094090d59c00e82213eddedaf9393a4953d2ae2703bcc6fafbe5fa72b</x:v>
+        <x:v>The 1814-1823 household records Pehr as head and Ingier as wife. It reports Pehr born 10 Feb 1791 and Ingier 20 Mar 1794; Pehr's baptism supplies the nearer 1790 birth year. Records: https://www.ancestry.com/search/collections/9731/records/91496907 ; https://www.ancestry.com/search/collections/9731/records/91496908</x:v>
       </x:c>
       <x:c r="F44" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="97" t="str">
-        <x:v>RECORD-1769-11-15_joshua-lane_hannah-tilton_marriage</x:v>
+        <x:v>S44</x:v>
       </x:c>
       <x:c r="B45" s="97" t="str">
-        <x:v>1769-11-15_joshua-lane_hannah-tilton_marriage.jpg</x:v>
-      </x:c>
-      <x:c r="C45" s="97" t="str"/>
-      <x:c r="D45" s="97" t="str"/>
+        <x:v>Pehr Erlandsson 1790 Hishult baptism</x:v>
+      </x:c>
+      <x:c r="C45" s="97" t="str">
+        <x:v>FamilySearch; Ancestry.com</x:v>
+      </x:c>
+      <x:c r="D45" s="97" t="str">
+        <x:v>14 FEB 1790</x:v>
+      </x:c>
       <x:c r="E45" s="97" t="str">
-        <x:v>9d1f204134ed96a42e5c7ddfe10e1265e03ae8c7af976cc6723f3836c6037d3e</x:v>
+        <x:v>Pehr was born 10 Feb and baptized 14 Feb 1790 at Hishult, son of Erland Pålsson and Bengta Pehrsdotter. https://www.ancestry.com/search/collections/60361/records/15528153</x:v>
       </x:c>
       <x:c r="F45" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="97" t="str">
-        <x:v>RECORD-1771-12-08_stephen-lane_nh-birth</x:v>
+        <x:v>S45</x:v>
       </x:c>
       <x:c r="B46" s="97" t="str">
-        <x:v>1771-12-08_stephen-lane_nh-birth.jpg</x:v>
-      </x:c>
-      <x:c r="C46" s="97" t="str"/>
-      <x:c r="D46" s="97" t="str"/>
+        <x:v>Ingier Hansdotter 1794 Hasslöv baptism</x:v>
+      </x:c>
+      <x:c r="C46" s="97" t="str">
+        <x:v>FamilySearch; Ancestry.com</x:v>
+      </x:c>
+      <x:c r="D46" s="97" t="str">
+        <x:v>23 MAR 1794</x:v>
+      </x:c>
       <x:c r="E46" s="97" t="str">
-        <x:v>4e983a0346e7c1b3d08b50d78c339d06a10d4ba9e23b8d7a2c932aa69343fd72</x:v>
+        <x:v>Ingier was born 20 Mar and baptized 23 Mar 1794 at Hasslöv, daughter of Hans Månsson and Maria Hansdotter. https://www.ancestry.com/search/collections/60361/records/11677925</x:v>
       </x:c>
       <x:c r="F46" s="97" t="str">
-        <x:v>preserved original or derivative record</x:v>
+        <x:v>cross-chat consolidation</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="97" t="str">
-        <x:v>RECORD-1774-02-26_levi-cook_birth-register</x:v>
+        <x:v>RECORD-1648-06-15_deborah-hopkins_birth-register</x:v>
       </x:c>
       <x:c r="B47" s="97" t="str">
-        <x:v>1774-02-26_levi-cook_birth-register.jpg</x:v>
+        <x:v>1648-06-15_deborah-hopkins_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C47" s="97" t="str"/>
       <x:c r="D47" s="97" t="str"/>
       <x:c r="E47" s="97" t="str">
-        <x:v>da32fa229e920c36321196b78361e9ea6df2ae57d08d34cf81279f9f727c5e26</x:v>
+        <x:v>4e6dd607655f9c2b251e3974596d63276178e76761116b370a8b16e0219f3f98</x:v>
       </x:c>
       <x:c r="F47" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5015,15 +5238,15 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="97" t="str">
-        <x:v>RECORD-1779-01-07_betsey-brown_birth-register</x:v>
+        <x:v>RECORD-1667-02-05_ephraim-doane_mary-knowles_marriage-register</x:v>
       </x:c>
       <x:c r="B48" s="97" t="str">
-        <x:v>1779-01-07_betsey-brown_birth-register.jpg</x:v>
+        <x:v>1667-02-05_ephraim-doane_mary-knowles_marriage-register.jpg</x:v>
       </x:c>
       <x:c r="C48" s="97" t="str"/>
       <x:c r="D48" s="97" t="str"/>
       <x:c r="E48" s="97" t="str">
-        <x:v>c43c3675e73e795d5d4ef90d64e64e746f1f9da1cf41ea0f2bbcddd01b50bfba</x:v>
+        <x:v>89ae0910e197b39bd902ca52685d144ab55193a340c5e6d3dbeb15a811487faa</x:v>
       </x:c>
       <x:c r="F48" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5031,15 +5254,15 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="97" t="str">
-        <x:v>RECORD-1794-07-24_levi-cook_betsey-brown_marriage-register</x:v>
+        <x:v>RECORD-1682-02-04_joshua-cook_birth-register</x:v>
       </x:c>
       <x:c r="B49" s="97" t="str">
-        <x:v>1794-07-24_levi-cook_betsey-brown_marriage-register.jpg</x:v>
+        <x:v>1682-02-04_joshua-cook_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C49" s="97" t="str"/>
       <x:c r="D49" s="97" t="str"/>
       <x:c r="E49" s="97" t="str">
-        <x:v>f3faf328a3ca886129787a18975b1c4892c5a5ed6bac9bebe5d6d4eb867f379f</x:v>
+        <x:v>726be1a255bf2abe13e2cdc2d149bcddf7dfb1702c466ab4e215d38133e9ea46</x:v>
       </x:c>
       <x:c r="F49" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5047,15 +5270,15 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="97" t="str">
-        <x:v>RECORD-1797-06-05_stephen-lane_lois-currier_marriage</x:v>
+        <x:v>RECORD-1682-04_patience-doane_birth-register</x:v>
       </x:c>
       <x:c r="B50" s="97" t="str">
-        <x:v>1797-06-05_stephen-lane_lois-currier_marriage.jpg</x:v>
+        <x:v>1682-04_patience-doane_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C50" s="97" t="str"/>
       <x:c r="D50" s="97" t="str"/>
       <x:c r="E50" s="97" t="str">
-        <x:v>6dd9495e06654018e796489a805f91471bd33329204c0b5171ee5425a898b280</x:v>
+        <x:v>c754af467f7252cd6952af7bc5948ce2ca5f77fdb7c7e60a6941088448c32e4a</x:v>
       </x:c>
       <x:c r="F50" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5063,15 +5286,15 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="97" t="str">
-        <x:v>RECORD-1807-02-03_mary-lane_nh-birth-card</x:v>
+        <x:v>RECORD-1696_joshua-lane_birth-record</x:v>
       </x:c>
       <x:c r="B51" s="97" t="str">
-        <x:v>1807-02-03_mary-lane_nh-birth-card.jpg</x:v>
+        <x:v>1696_joshua-lane_birth-record.jpg</x:v>
       </x:c>
       <x:c r="C51" s="97" t="str"/>
       <x:c r="D51" s="97" t="str"/>
       <x:c r="E51" s="97" t="str">
-        <x:v>54e52adccc86fbb08e9fd36c8ad80efbb130eb34178bf7f4cae9bfe9fae15351</x:v>
+        <x:v>23c17bccf0b93d5ca970ddc6458dc14f264e129c5650c13a9e613dc57e94371e</x:v>
       </x:c>
       <x:c r="F51" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5079,15 +5302,15 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="97" t="str">
-        <x:v>RECORD-1840-09-16_stephen-lane_will</x:v>
+        <x:v>RECORD-1717_joshua-lane_bathsheba-robie_marriage-record</x:v>
       </x:c>
       <x:c r="B52" s="97" t="str">
-        <x:v>1840-09-16_stephen-lane_will.jpg</x:v>
+        <x:v>1717_joshua-lane_bathsheba-robie_marriage-record.jpg</x:v>
       </x:c>
       <x:c r="C52" s="97" t="str"/>
       <x:c r="D52" s="97" t="str"/>
       <x:c r="E52" s="97" t="str">
-        <x:v>773c3a78efbeac6efc48f53d6d01f7556aade77197bb59cb85265cb67c5b4f99</x:v>
+        <x:v>15e63b00090b98e21bb4ae4d28cc0d2a620bbe75946c63efe681f5b512fb6b9c</x:v>
       </x:c>
       <x:c r="F52" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5095,15 +5318,15 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="97" t="str">
-        <x:v>RECORD-1841-05-05_stephen-lane_probate-letters</x:v>
+        <x:v>RECORD-1718_samuel-lane_birth-record</x:v>
       </x:c>
       <x:c r="B53" s="97" t="str">
-        <x:v>1841-05-05_stephen-lane_probate-letters.jpg</x:v>
+        <x:v>1718_samuel-lane_birth-record.jpg</x:v>
       </x:c>
       <x:c r="C53" s="97" t="str"/>
       <x:c r="D53" s="97" t="str"/>
       <x:c r="E53" s="97" t="str">
-        <x:v>dca2ab0c7608fe5ca72e5d18e3bb9d920173d4535609fca51f115c9de62c2c04</x:v>
+        <x:v>0200f2252b3392cf2fa2ecb3d58b9ddef31b998ce5d76ef552bfab2ee7eda016</x:v>
       </x:c>
       <x:c r="F53" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5111,15 +5334,15 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="97" t="str">
-        <x:v>RECORD-1846-10-30_levi-cook_will_genesee</x:v>
+        <x:v>RECORD-1722_mary-james_birth-record</x:v>
       </x:c>
       <x:c r="B54" s="97" t="str">
-        <x:v>1846-10-30_levi-cook_will_genesee.jpg</x:v>
+        <x:v>1722_mary-james_birth-record.jpg</x:v>
       </x:c>
       <x:c r="C54" s="97" t="str"/>
       <x:c r="D54" s="97" t="str"/>
       <x:c r="E54" s="97" t="str">
-        <x:v>ca99721390ba6f33558e3a0ce805f614dabed6ee6aab6dce762506bf16f00235</x:v>
+        <x:v>189899f04cbc5dc801896487041938515771118dabdb1af87ed6662a4f6ffcd9</x:v>
       </x:c>
       <x:c r="F54" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5127,15 +5350,15 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="97" t="str">
-        <x:v>RECORD-1862_peter-william-mcnaughton_civil-war-town-register</x:v>
+        <x:v>RECORD-1741-12-24_samuel-lane_mary-james_marriage</x:v>
       </x:c>
       <x:c r="B55" s="97" t="str">
-        <x:v>1862_peter-william-mcnaughton_civil-war-town-register.jpg</x:v>
+        <x:v>1741-12-24_samuel-lane_mary-james_marriage.jpg</x:v>
       </x:c>
       <x:c r="C55" s="97" t="str"/>
       <x:c r="D55" s="97" t="str"/>
       <x:c r="E55" s="97" t="str">
-        <x:v>7e767cf4e9ce3792ea381e5dcea992eade9ac9d7e361eae2e6927ed41b52a9b4</x:v>
+        <x:v>fd6d017aaaa9f3c51bd77b7c6a0a007e08a6b28b3eacd4323314c75ced5f61b4</x:v>
       </x:c>
       <x:c r="F55" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5143,15 +5366,15 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="97" t="str">
-        <x:v>RECORD-1868_relief-mcnaughton_dependent-pension-numerical-index</x:v>
+        <x:v>RECORD-1748-02-09_joshua-lane_nh-birth</x:v>
       </x:c>
       <x:c r="B56" s="97" t="str">
-        <x:v>1868_relief-mcnaughton_dependent-pension-numerical-index.jpg</x:v>
+        <x:v>1748-02-09_joshua-lane_nh-birth.jpg</x:v>
       </x:c>
       <x:c r="C56" s="97" t="str"/>
       <x:c r="D56" s="97" t="str"/>
       <x:c r="E56" s="97" t="str">
-        <x:v>122349eb44bcbf808eaa9d841bec77cb9b433ff01d7b88dd9f862441a237ed6e</x:v>
+        <x:v>8b75cc1094090d59c00e82213eddedaf9393a4953d2ae2703bcc6fafbe5fa72b</x:v>
       </x:c>
       <x:c r="F56" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5159,15 +5382,15 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="97" t="str">
-        <x:v>RECORD-1882-08-21_henry-vollmer_arrival-main</x:v>
+        <x:v>RECORD-1769-11-15_joshua-lane_hannah-tilton_marriage</x:v>
       </x:c>
       <x:c r="B57" s="97" t="str">
-        <x:v>1882-08-21_henry-vollmer_arrival-main.jpg</x:v>
+        <x:v>1769-11-15_joshua-lane_hannah-tilton_marriage.jpg</x:v>
       </x:c>
       <x:c r="C57" s="97" t="str"/>
       <x:c r="D57" s="97" t="str"/>
       <x:c r="E57" s="97" t="str">
-        <x:v>319186b29241957f4be18e4f2c4d350679c5b0c36f6ee3330ba90a62dbca0b24</x:v>
+        <x:v>9d1f204134ed96a42e5c7ddfe10e1265e03ae8c7af976cc6723f3836c6037d3e</x:v>
       </x:c>
       <x:c r="F57" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5175,15 +5398,15 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="97" t="str">
-        <x:v>RECORD-1882-08-21_vollmer-family_arrival-main_page-0289</x:v>
+        <x:v>RECORD-1771-12-08_stephen-lane_nh-birth</x:v>
       </x:c>
       <x:c r="B58" s="97" t="str">
-        <x:v>1882-08-21_vollmer-family_arrival-main_page-0289.jpg</x:v>
+        <x:v>1771-12-08_stephen-lane_nh-birth.jpg</x:v>
       </x:c>
       <x:c r="C58" s="97" t="str"/>
       <x:c r="D58" s="97" t="str"/>
       <x:c r="E58" s="97" t="str">
-        <x:v>747649d753285ae52234547090101c60660612500bc3132a35f57b13a0ce9e11</x:v>
+        <x:v>4e983a0346e7c1b3d08b50d78c339d06a10d4ba9e23b8d7a2c932aa69343fd72</x:v>
       </x:c>
       <x:c r="F58" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5191,15 +5414,15 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="97" t="str">
-        <x:v>RECORD-1883-08-12_themes-pepper_anna-stelling_marriage-certificate</x:v>
+        <x:v>RECORD-1774-02-26_levi-cook_birth-register</x:v>
       </x:c>
       <x:c r="B59" s="97" t="str">
-        <x:v>1883-08-12_themes-pepper_anna-stelling_marriage-certificate.pdf</x:v>
+        <x:v>1774-02-26_levi-cook_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C59" s="97" t="str"/>
       <x:c r="D59" s="97" t="str"/>
       <x:c r="E59" s="97" t="str">
-        <x:v>2a89c49df0051c74dbc241741e7b75dbabeff093782428e3a3b82cd002de44bd</x:v>
+        <x:v>da32fa229e920c36321196b78361e9ea6df2ae57d08d34cf81279f9f727c5e26</x:v>
       </x:c>
       <x:c r="F59" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5207,15 +5430,15 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="97" t="str">
-        <x:v>RECORD-1884-03-14_female-pepper_birth-certificate</x:v>
+        <x:v>RECORD-1779-01-07_betsey-brown_birth-register</x:v>
       </x:c>
       <x:c r="B60" s="97" t="str">
-        <x:v>1884-03-14_female-pepper_birth-certificate.pdf</x:v>
+        <x:v>1779-01-07_betsey-brown_birth-register.jpg</x:v>
       </x:c>
       <x:c r="C60" s="97" t="str"/>
       <x:c r="D60" s="97" t="str"/>
       <x:c r="E60" s="97" t="str">
-        <x:v>d457e8478154d51688ddd777101aee2501f89ef8f4515eab0a8cf431076d7180</x:v>
+        <x:v>c43c3675e73e795d5d4ef90d64e64e746f1f9da1cf41ea0f2bbcddd01b50bfba</x:v>
       </x:c>
       <x:c r="F60" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5223,15 +5446,15 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="97" t="str">
-        <x:v>RECORD-1892_henry-vollmer_ny-state-census</x:v>
+        <x:v>RECORD-1794-07-24_levi-cook_betsey-brown_marriage-register</x:v>
       </x:c>
       <x:c r="B61" s="97" t="str">
-        <x:v>1892_henry-vollmer_ny-state-census.jpg</x:v>
+        <x:v>1794-07-24_levi-cook_betsey-brown_marriage-register.jpg</x:v>
       </x:c>
       <x:c r="C61" s="97" t="str"/>
       <x:c r="D61" s="97" t="str"/>
       <x:c r="E61" s="97" t="str">
-        <x:v>480f9a9c4d79a918392467e6ebf758452a8d200ad3692cb7f436a4654d688421</x:v>
+        <x:v>f3faf328a3ca886129787a18975b1c4892c5a5ed6bac9bebe5d6d4eb867f379f</x:v>
       </x:c>
       <x:c r="F61" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5239,15 +5462,15 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="97" t="str">
-        <x:v>RECORD-1896_mary-a-mcnaughton_widow-pension-index</x:v>
+        <x:v>RECORD-1797-06-05_stephen-lane_lois-currier_marriage</x:v>
       </x:c>
       <x:c r="B62" s="97" t="str">
-        <x:v>1896_mary-a-mcnaughton_widow-pension-index.jpg</x:v>
+        <x:v>1797-06-05_stephen-lane_lois-currier_marriage.jpg</x:v>
       </x:c>
       <x:c r="C62" s="97" t="str"/>
       <x:c r="D62" s="97" t="str"/>
       <x:c r="E62" s="97" t="str">
-        <x:v>14d064d694dc478f36bb570e78e29368a0259693dfb7217c05975c508bd01db8</x:v>
+        <x:v>6dd9495e06654018e796489a805f91471bd33329204c0b5171ee5425a898b280</x:v>
       </x:c>
       <x:c r="F62" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5255,15 +5478,15 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="97" t="str">
-        <x:v>RECORD-1901_mayflower-descendant-vol3_john-doane-will</x:v>
+        <x:v>RECORD-1807-02-03_mary-lane_nh-birth-card</x:v>
       </x:c>
       <x:c r="B63" s="97" t="str">
-        <x:v>1901_mayflower-descendant-vol3_john-doane-will.pdf</x:v>
+        <x:v>1807-02-03_mary-lane_nh-birth-card.jpg</x:v>
       </x:c>
       <x:c r="C63" s="97" t="str"/>
       <x:c r="D63" s="97" t="str"/>
       <x:c r="E63" s="97" t="str">
-        <x:v>4d7d359130d69d3db9e5ebdec3f22833c097c0e9dad4e5602047f370bd057518</x:v>
+        <x:v>54e52adccc86fbb08e9fd36c8ad80efbb130eb34178bf7f4cae9bfe9fae15351</x:v>
       </x:c>
       <x:c r="F63" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5271,15 +5494,15 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="97" t="str">
-        <x:v>RECORD-1904_mayflower-descendant-vol6_eastham-vital-records</x:v>
+        <x:v>RECORD-1840-09-16_stephen-lane_will</x:v>
       </x:c>
       <x:c r="B64" s="97" t="str">
-        <x:v>1904_mayflower-descendant-vol6_eastham-vital-records.pdf</x:v>
+        <x:v>1840-09-16_stephen-lane_will.jpg</x:v>
       </x:c>
       <x:c r="C64" s="97" t="str"/>
       <x:c r="D64" s="97" t="str"/>
       <x:c r="E64" s="97" t="str">
-        <x:v>105a13412229bb5489c9e245faa82209405ec7199e5fe371dc17a09d1351ba3a</x:v>
+        <x:v>773c3a78efbeac6efc48f53d6d01f7556aade77197bb59cb85265cb67c5b4f99</x:v>
       </x:c>
       <x:c r="F64" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5287,15 +5510,15 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="97" t="str">
-        <x:v>RECORD-1905-08-05_henry-jj-vollmer_marriage-certificate</x:v>
+        <x:v>RECORD-1841-05-05_stephen-lane_probate-letters</x:v>
       </x:c>
       <x:c r="B65" s="97" t="str">
-        <x:v>1905-08-05_henry-jj-vollmer_marriage-certificate.pdf</x:v>
+        <x:v>1841-05-05_stephen-lane_probate-letters.jpg</x:v>
       </x:c>
       <x:c r="C65" s="97" t="str"/>
       <x:c r="D65" s="97" t="str"/>
       <x:c r="E65" s="97" t="str">
-        <x:v>59b537c81462fcba56c9827e5a015dacefafd451442735b8db6a37fcccabe2a9</x:v>
+        <x:v>dca2ab0c7608fe5ca72e5d18e3bb9d920173d4535609fca51f115c9de62c2c04</x:v>
       </x:c>
       <x:c r="F65" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5303,15 +5526,15 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="97" t="str">
-        <x:v>RECORD-1910_frederick-carrie-doris-andrew-marsh_us-census</x:v>
+        <x:v>RECORD-1846-10-30_levi-cook_will_genesee</x:v>
       </x:c>
       <x:c r="B66" s="97" t="str">
-        <x:v>1910_frederick-carrie-doris-andrew-marsh_us-census.jpg</x:v>
+        <x:v>1846-10-30_levi-cook_will_genesee.jpg</x:v>
       </x:c>
       <x:c r="C66" s="97" t="str"/>
       <x:c r="D66" s="97" t="str"/>
       <x:c r="E66" s="97" t="str">
-        <x:v>88afa43f7bb90fc8248f9158ccae50b081e820e9e690022c2ec446434ce47bf4</x:v>
+        <x:v>ca99721390ba6f33558e3a0ce805f614dabed6ee6aab6dce762506bf16f00235</x:v>
       </x:c>
       <x:c r="F66" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5319,15 +5542,15 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="97" t="str">
-        <x:v>RECORD-1910_henry-madie-charles-vollmer_us-census</x:v>
+        <x:v>RECORD-1862_peter-william-mcnaughton_civil-war-town-register</x:v>
       </x:c>
       <x:c r="B67" s="97" t="str">
-        <x:v>1910_henry-madie-charles-vollmer_us-census.jpg</x:v>
+        <x:v>1862_peter-william-mcnaughton_civil-war-town-register.jpg</x:v>
       </x:c>
       <x:c r="C67" s="97" t="str"/>
       <x:c r="D67" s="97" t="str"/>
       <x:c r="E67" s="97" t="str">
-        <x:v>5506a666f811c403bc06da8594751a45791c6f2f60ec7d61bf02be7d70f5bade</x:v>
+        <x:v>7e767cf4e9ce3792ea381e5dcea992eade9ac9d7e361eae2e6927ed41b52a9b4</x:v>
       </x:c>
       <x:c r="F67" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5335,15 +5558,15 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="97" t="str">
-        <x:v>RECORD-1917-03-10_frederick-g-vollmer_death-certificate</x:v>
+        <x:v>RECORD-1868_relief-mcnaughton_dependent-pension-numerical-index</x:v>
       </x:c>
       <x:c r="B68" s="97" t="str">
-        <x:v>1917-03-10_frederick-g-vollmer_death-certificate.pdf</x:v>
+        <x:v>1868_relief-mcnaughton_dependent-pension-numerical-index.jpg</x:v>
       </x:c>
       <x:c r="C68" s="97" t="str"/>
       <x:c r="D68" s="97" t="str"/>
       <x:c r="E68" s="97" t="str">
-        <x:v>eb970b4f9f3954c566fe8b3cd5d245162172d247dfc39f93aec396307c88bfc1</x:v>
+        <x:v>122349eb44bcbf808eaa9d841bec77cb9b433ff01d7b88dd9f862441a237ed6e</x:v>
       </x:c>
       <x:c r="F68" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5351,15 +5574,15 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="97" t="str">
-        <x:v>RECORD-1918_henry-john-joseph-volmer_wwi-draft-card</x:v>
+        <x:v>RECORD-1882-08-21_henry-vollmer_arrival-main</x:v>
       </x:c>
       <x:c r="B69" s="97" t="str">
-        <x:v>1918_henry-john-joseph-volmer_wwi-draft-card.jpg</x:v>
+        <x:v>1882-08-21_henry-vollmer_arrival-main.jpg</x:v>
       </x:c>
       <x:c r="C69" s="97" t="str"/>
       <x:c r="D69" s="97" t="str"/>
       <x:c r="E69" s="97" t="str">
-        <x:v>6a929ffb761b504b27bc2cdf2f905fc2ea0b7351cd0554fdd8f38256494367f6</x:v>
+        <x:v>319186b29241957f4be18e4f2c4d350679c5b0c36f6ee3330ba90a62dbca0b24</x:v>
       </x:c>
       <x:c r="F69" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5367,15 +5590,15 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="97" t="str">
-        <x:v>RECORD-1919-01-03_madie-vollmer_death-certificate</x:v>
+        <x:v>RECORD-1882-08-21_vollmer-family_arrival-main_page-0289</x:v>
       </x:c>
       <x:c r="B70" s="97" t="str">
-        <x:v>1919-01-03_madie-vollmer_death-certificate.pdf</x:v>
+        <x:v>1882-08-21_vollmer-family_arrival-main_page-0289.jpg</x:v>
       </x:c>
       <x:c r="C70" s="97" t="str"/>
       <x:c r="D70" s="97" t="str"/>
       <x:c r="E70" s="97" t="str">
-        <x:v>8f8be8c3cb340d5032a2d61e4ed5b578e782c0176054592aee8e48abe1174734</x:v>
+        <x:v>747649d753285ae52234547090101c60660612500bc3132a35f57b13a0ce9e11</x:v>
       </x:c>
       <x:c r="F70" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5383,15 +5606,15 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="97" t="str">
-        <x:v>RECORD-1919-12-17_mary-mcnaughton_ny-death-index</x:v>
+        <x:v>RECORD-1883-08-12_themes-pepper_anna-stelling_marriage-certificate</x:v>
       </x:c>
       <x:c r="B71" s="97" t="str">
-        <x:v>1919-12-17_mary-mcnaughton_ny-death-index.jpg</x:v>
+        <x:v>1883-08-12_themes-pepper_anna-stelling_marriage-certificate.pdf</x:v>
       </x:c>
       <x:c r="C71" s="97" t="str"/>
       <x:c r="D71" s="97" t="str"/>
       <x:c r="E71" s="97" t="str">
-        <x:v>2ccad7fd75e95b52575500ee7ff48c3285db4b0d6680654727bf58c704044b3d</x:v>
+        <x:v>2a89c49df0051c74dbc241741e7b75dbabeff093782428e3a3b82cd002de44bd</x:v>
       </x:c>
       <x:c r="F71" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5399,15 +5622,15 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="97" t="str">
-        <x:v>RECORD-1940-10-16_charles-frederick-vollmer_wwii-draft-card</x:v>
+        <x:v>RECORD-1884-03-14_female-pepper_birth-certificate</x:v>
       </x:c>
       <x:c r="B72" s="97" t="str">
-        <x:v>1940-10-16_charles-frederick-vollmer_wwii-draft-card.jpg</x:v>
+        <x:v>1884-03-14_female-pepper_birth-certificate.pdf</x:v>
       </x:c>
       <x:c r="C72" s="97" t="str"/>
       <x:c r="D72" s="97" t="str"/>
       <x:c r="E72" s="97" t="str">
-        <x:v>e755e1f176b897bc6ea96a2ad3bf6697b9634d65f315c438ebefa97638897160</x:v>
+        <x:v>d457e8478154d51688ddd777101aee2501f89ef8f4515eab0a8cf431076d7180</x:v>
       </x:c>
       <x:c r="F72" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5415,15 +5638,15 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="97" t="str">
-        <x:v>RECORD-1940_charles-doris-henry-vollmer_us-census</x:v>
+        <x:v>RECORD-1892_henry-vollmer_ny-state-census</x:v>
       </x:c>
       <x:c r="B73" s="97" t="str">
-        <x:v>1940_charles-doris-henry-vollmer_us-census.jpg</x:v>
+        <x:v>1892_henry-vollmer_ny-state-census.jpg</x:v>
       </x:c>
       <x:c r="C73" s="97" t="str"/>
       <x:c r="D73" s="97" t="str"/>
       <x:c r="E73" s="97" t="str">
-        <x:v>408d8f6dd3a769e32af16d8cc59f762113000942a482dafa1b9ea01431c71ebb</x:v>
+        <x:v>480f9a9c4d79a918392467e6ebf758452a8d200ad3692cb7f436a4654d688421</x:v>
       </x:c>
       <x:c r="F73" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5431,15 +5654,15 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="97" t="str">
-        <x:v>RECORD-1950_william-alice-mary-thoren_us-census</x:v>
+        <x:v>RECORD-1896_mary-a-mcnaughton_widow-pension-index</x:v>
       </x:c>
       <x:c r="B74" s="97" t="str">
-        <x:v>1950_william-alice-mary-thoren_us-census.jpg</x:v>
+        <x:v>1896_mary-a-mcnaughton_widow-pension-index.jpg</x:v>
       </x:c>
       <x:c r="C74" s="97" t="str"/>
       <x:c r="D74" s="97" t="str"/>
       <x:c r="E74" s="97" t="str">
-        <x:v>f7e7dde0bcc80447fef0ed66c9699bf2477115f8ea97a2d464724c28c4bb7db5</x:v>
+        <x:v>14d064d694dc478f36bb570e78e29368a0259693dfb7217c05975c508bd01db8</x:v>
       </x:c>
       <x:c r="F74" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5447,15 +5670,15 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="97" t="str">
-        <x:v>RECORD-giles-hopkins_17th-century-records_pilgrim-hall</x:v>
+        <x:v>RECORD-1901_mayflower-descendant-vol3_john-doane-will</x:v>
       </x:c>
       <x:c r="B75" s="97" t="str">
-        <x:v>giles-hopkins_17th-century-records_pilgrim-hall.pdf</x:v>
+        <x:v>1901_mayflower-descendant-vol3_john-doane-will.pdf</x:v>
       </x:c>
       <x:c r="C75" s="97" t="str"/>
       <x:c r="D75" s="97" t="str"/>
       <x:c r="E75" s="97" t="str">
-        <x:v>1dbca70bd43b7dd62a3e12bc3b9ee230d8baa0dd37b80cc53ab48ec757763e01</x:v>
+        <x:v>4d7d359130d69d3db9e5ebdec3f22833c097c0e9dad4e5602047f370bd057518</x:v>
       </x:c>
       <x:c r="F75" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5463,15 +5686,15 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="97" t="str">
-        <x:v>RECORD-plymouth-colony-records-vol1_1639-marriage</x:v>
+        <x:v>RECORD-1904_mayflower-descendant-vol6_eastham-vital-records</x:v>
       </x:c>
       <x:c r="B76" s="97" t="str">
-        <x:v>plymouth-colony-records-vol1_1639-marriage.pdf</x:v>
+        <x:v>1904_mayflower-descendant-vol6_eastham-vital-records.pdf</x:v>
       </x:c>
       <x:c r="C76" s="97" t="str"/>
       <x:c r="D76" s="97" t="str"/>
       <x:c r="E76" s="97" t="str">
-        <x:v>243bba40de735bf7deedf4046c40f190526cb1c5cc891ef97a348248067d6cbd</x:v>
+        <x:v>105a13412229bb5489c9e245faa82209405ec7199e5fe371dc17a09d1351ba3a</x:v>
       </x:c>
       <x:c r="F76" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
@@ -5479,24 +5702,216 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="97" t="str">
-        <x:v>RECORD-relief-mcnaughton_mother-pension-index</x:v>
+        <x:v>RECORD-1905-08-05_henry-jj-vollmer_marriage-certificate</x:v>
       </x:c>
       <x:c r="B77" s="97" t="str">
-        <x:v>relief-mcnaughton_mother-pension-index.jpg</x:v>
+        <x:v>1905-08-05_henry-jj-vollmer_marriage-certificate.pdf</x:v>
       </x:c>
       <x:c r="C77" s="97" t="str"/>
       <x:c r="D77" s="97" t="str"/>
       <x:c r="E77" s="97" t="str">
+        <x:v>59b537c81462fcba56c9827e5a015dacefafd451442735b8db6a37fcccabe2a9</x:v>
+      </x:c>
+      <x:c r="F77" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="97" t="str">
+        <x:v>RECORD-1910_frederick-carrie-doris-andrew-marsh_us-census</x:v>
+      </x:c>
+      <x:c r="B78" s="97" t="str">
+        <x:v>1910_frederick-carrie-doris-andrew-marsh_us-census.jpg</x:v>
+      </x:c>
+      <x:c r="C78" s="97" t="str"/>
+      <x:c r="D78" s="97" t="str"/>
+      <x:c r="E78" s="97" t="str">
+        <x:v>88afa43f7bb90fc8248f9158ccae50b081e820e9e690022c2ec446434ce47bf4</x:v>
+      </x:c>
+      <x:c r="F78" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="97" t="str">
+        <x:v>RECORD-1910_henry-madie-charles-vollmer_us-census</x:v>
+      </x:c>
+      <x:c r="B79" s="97" t="str">
+        <x:v>1910_henry-madie-charles-vollmer_us-census.jpg</x:v>
+      </x:c>
+      <x:c r="C79" s="97" t="str"/>
+      <x:c r="D79" s="97" t="str"/>
+      <x:c r="E79" s="97" t="str">
+        <x:v>5506a666f811c403bc06da8594751a45791c6f2f60ec7d61bf02be7d70f5bade</x:v>
+      </x:c>
+      <x:c r="F79" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="97" t="str">
+        <x:v>RECORD-1917-03-10_frederick-g-vollmer_death-certificate</x:v>
+      </x:c>
+      <x:c r="B80" s="97" t="str">
+        <x:v>1917-03-10_frederick-g-vollmer_death-certificate.pdf</x:v>
+      </x:c>
+      <x:c r="C80" s="97" t="str"/>
+      <x:c r="D80" s="97" t="str"/>
+      <x:c r="E80" s="97" t="str">
+        <x:v>eb970b4f9f3954c566fe8b3cd5d245162172d247dfc39f93aec396307c88bfc1</x:v>
+      </x:c>
+      <x:c r="F80" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="97" t="str">
+        <x:v>RECORD-1918_henry-john-joseph-volmer_wwi-draft-card</x:v>
+      </x:c>
+      <x:c r="B81" s="97" t="str">
+        <x:v>1918_henry-john-joseph-volmer_wwi-draft-card.jpg</x:v>
+      </x:c>
+      <x:c r="C81" s="97" t="str"/>
+      <x:c r="D81" s="97" t="str"/>
+      <x:c r="E81" s="97" t="str">
+        <x:v>6a929ffb761b504b27bc2cdf2f905fc2ea0b7351cd0554fdd8f38256494367f6</x:v>
+      </x:c>
+      <x:c r="F81" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="97" t="str">
+        <x:v>RECORD-1919-01-03_madie-vollmer_death-certificate</x:v>
+      </x:c>
+      <x:c r="B82" s="97" t="str">
+        <x:v>1919-01-03_madie-vollmer_death-certificate.pdf</x:v>
+      </x:c>
+      <x:c r="C82" s="97" t="str"/>
+      <x:c r="D82" s="97" t="str"/>
+      <x:c r="E82" s="97" t="str">
+        <x:v>8f8be8c3cb340d5032a2d61e4ed5b578e782c0176054592aee8e48abe1174734</x:v>
+      </x:c>
+      <x:c r="F82" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="97" t="str">
+        <x:v>RECORD-1919-12-17_mary-mcnaughton_ny-death-index</x:v>
+      </x:c>
+      <x:c r="B83" s="97" t="str">
+        <x:v>1919-12-17_mary-mcnaughton_ny-death-index.jpg</x:v>
+      </x:c>
+      <x:c r="C83" s="97" t="str"/>
+      <x:c r="D83" s="97" t="str"/>
+      <x:c r="E83" s="97" t="str">
+        <x:v>2ccad7fd75e95b52575500ee7ff48c3285db4b0d6680654727bf58c704044b3d</x:v>
+      </x:c>
+      <x:c r="F83" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="97" t="str">
+        <x:v>RECORD-1940-10-16_charles-frederick-vollmer_wwii-draft-card</x:v>
+      </x:c>
+      <x:c r="B84" s="97" t="str">
+        <x:v>1940-10-16_charles-frederick-vollmer_wwii-draft-card.jpg</x:v>
+      </x:c>
+      <x:c r="C84" s="97" t="str"/>
+      <x:c r="D84" s="97" t="str"/>
+      <x:c r="E84" s="97" t="str">
+        <x:v>e755e1f176b897bc6ea96a2ad3bf6697b9634d65f315c438ebefa97638897160</x:v>
+      </x:c>
+      <x:c r="F84" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="97" t="str">
+        <x:v>RECORD-1940_charles-doris-henry-vollmer_us-census</x:v>
+      </x:c>
+      <x:c r="B85" s="97" t="str">
+        <x:v>1940_charles-doris-henry-vollmer_us-census.jpg</x:v>
+      </x:c>
+      <x:c r="C85" s="97" t="str"/>
+      <x:c r="D85" s="97" t="str"/>
+      <x:c r="E85" s="97" t="str">
+        <x:v>408d8f6dd3a769e32af16d8cc59f762113000942a482dafa1b9ea01431c71ebb</x:v>
+      </x:c>
+      <x:c r="F85" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="97" t="str">
+        <x:v>RECORD-1950_william-alice-mary-thoren_us-census</x:v>
+      </x:c>
+      <x:c r="B86" s="97" t="str">
+        <x:v>1950_william-alice-mary-thoren_us-census.jpg</x:v>
+      </x:c>
+      <x:c r="C86" s="97" t="str"/>
+      <x:c r="D86" s="97" t="str"/>
+      <x:c r="E86" s="97" t="str">
+        <x:v>f7e7dde0bcc80447fef0ed66c9699bf2477115f8ea97a2d464724c28c4bb7db5</x:v>
+      </x:c>
+      <x:c r="F86" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="97" t="str">
+        <x:v>RECORD-giles-hopkins_17th-century-records_pilgrim-hall</x:v>
+      </x:c>
+      <x:c r="B87" s="97" t="str">
+        <x:v>giles-hopkins_17th-century-records_pilgrim-hall.pdf</x:v>
+      </x:c>
+      <x:c r="C87" s="97" t="str"/>
+      <x:c r="D87" s="97" t="str"/>
+      <x:c r="E87" s="97" t="str">
+        <x:v>1dbca70bd43b7dd62a3e12bc3b9ee230d8baa0dd37b80cc53ab48ec757763e01</x:v>
+      </x:c>
+      <x:c r="F87" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="97" t="str">
+        <x:v>RECORD-plymouth-colony-records-vol1_1639-marriage</x:v>
+      </x:c>
+      <x:c r="B88" s="97" t="str">
+        <x:v>plymouth-colony-records-vol1_1639-marriage.pdf</x:v>
+      </x:c>
+      <x:c r="C88" s="97" t="str"/>
+      <x:c r="D88" s="97" t="str"/>
+      <x:c r="E88" s="97" t="str">
+        <x:v>243bba40de735bf7deedf4046c40f190526cb1c5cc891ef97a348248067d6cbd</x:v>
+      </x:c>
+      <x:c r="F88" s="97" t="str">
+        <x:v>preserved original or derivative record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="97" t="str">
+        <x:v>RECORD-relief-mcnaughton_mother-pension-index</x:v>
+      </x:c>
+      <x:c r="B89" s="97" t="str">
+        <x:v>relief-mcnaughton_mother-pension-index.jpg</x:v>
+      </x:c>
+      <x:c r="C89" s="97" t="str"/>
+      <x:c r="D89" s="97" t="str"/>
+      <x:c r="E89" s="97" t="str">
         <x:v>4c481d5447084325803d01ea3fb19e1485b4d96fd24cc06c3c83ed32580e90f7</x:v>
       </x:c>
-      <x:c r="F77" s="97" t="str">
+      <x:c r="F89" s="97" t="str">
         <x:v>preserved original or derivative record</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R029ba46886db4a0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9f5adcf273442f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5564,15 +5979,15 @@
         <x:v>Individuals</x:v>
       </x:c>
       <x:c r="B5" s="92" t="n">
-        <x:f>COUNTA('Consolidated People'!$A$2:$A$311)</x:f>
-        <x:v>310</x:v>
+        <x:f>COUNTA('Consolidated People'!$A$2:$A$328)</x:f>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="C5" s="80"/>
       <x:c r="D5" s="94" t="str">
         <x:v>Jan is Fredric's biological mother</x:v>
       </x:c>
       <x:c r="E5" s="95" t="str">
-        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$311,"Jan Muller Vollmer")=1,"Confirmed","Review")</x:f>
+        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$328,"Jan Muller Vollmer")=1,"Confirmed","Review")</x:f>
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
@@ -5584,19 +5999,19 @@
         <x:v>Families</x:v>
       </x:c>
       <x:c r="B6" s="92" t="n">
-        <x:f>COUNTA('Consolidated Families'!$A$2:$A$146)</x:f>
-        <x:v>145</x:v>
+        <x:f>COUNTA('Consolidated Families'!$A$2:$A$155)</x:f>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C6" s="80"/>
       <x:c r="D6" s="94" t="str">
         <x:v>Mary Alice Thoren identity and parents</x:v>
       </x:c>
       <x:c r="E6" s="95" t="str">
-        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$311,"Mary Alice Thoren")=1,"Confirmed","Review")</x:f>
+        <x:f>IF(COUNTIF('Consolidated People'!$B$2:$B$328,"Mary Alice Thoren")=1,"Confirmed","Review")</x:f>
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="F6" s="94" t="str">
-        <x:v>Port Townsend birthplace; William J. Thoren and Alice Gallaher parent links; first marriage to Henry recorded</x:v>
+        <x:v>Port Townsend birthplace; William and Alice parent links; William's proven Swedish ancestry added; Alice's parents remain unresolved</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -5604,8 +6019,8 @@
         <x:v>GEDCOM source records</x:v>
       </x:c>
       <x:c r="B7" s="92" t="n">
-        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$34)</x:f>
-        <x:v>33</x:v>
+        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$46)</x:f>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C7" s="80"/>
       <x:c r="D7" s="94" t="str">
@@ -5623,8 +6038,8 @@
         <x:v>Source and record inventory items</x:v>
       </x:c>
       <x:c r="B8" s="92" t="n">
-        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$77)</x:f>
-        <x:v>76</x:v>
+        <x:f>COUNTA('Consolidated Sources'!$A$2:$A$89)</x:f>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="C8" s="80"/>
       <x:c r="D8" s="94" t="str">
@@ -5687,7 +6102,7 @@
         <x:v>Canonical tree structure</x:v>
       </x:c>
       <x:c r="C12" s="97" t="n">
-        <x:v>310</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="D12" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree.ged</x:v>
@@ -5707,7 +6122,7 @@
         <x:v>Structured mirror</x:v>
       </x:c>
       <x:c r="C13" s="97" t="n">
-        <x:v>310</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="D13" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_Canonical_Data.json</x:v>
@@ -5727,7 +6142,7 @@
         <x:v>Person-level audit</x:v>
       </x:c>
       <x:c r="C14" s="97" t="n">
-        <x:v>310</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="D14" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_People.csv</x:v>
@@ -5747,7 +6162,7 @@
         <x:v>Family-level audit</x:v>
       </x:c>
       <x:c r="C15" s="97" t="n">
-        <x:v>145</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="D15" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_Families.csv</x:v>
@@ -5767,7 +6182,7 @@
         <x:v>Citation and record index</x:v>
       </x:c>
       <x:c r="C16" s="97" t="n">
-        <x:v>76</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D16" s="97" t="str">
         <x:v>Fredric_Vollmer_Complete_Family_Tree_Source_Inventory.csv</x:v>
@@ -5776,7 +6191,7 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="F16" s="97" t="str">
-        <x:v>Includes 33 GEDCOM sources and 43 preserved record files</x:v>
+        <x:v>Includes 45 GEDCOM sources and 43 preserved record files</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
@@ -17602,7 +18017,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95657ae8b9b34f09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19af7ef07b2f4025"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21729,7 +22144,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f66bbbe0868449e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25fa7e2358244f4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24658,7 +25073,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb61ca122ff65431b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78516096c5884c7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25012,7 +25427,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23624991a5784c13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22b81a593faa45f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25206,7 +25621,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48e9016022654a7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra871cf7d62fb40bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25684,7 +26099,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re747d8b77caf4964"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba16bd47f5d5485b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26767,7 +27182,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41c4f7e1ecbc4482"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb847224604884181"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35483,25 +35898,29 @@
         <x:v>I336</x:v>
       </x:c>
       <x:c r="B310" s="97" t="str">
-        <x:v>William J Thoren</x:v>
+        <x:v>William John Thoren</x:v>
       </x:c>
       <x:c r="C310" s="97" t="str">
         <x:v>M</x:v>
       </x:c>
       <x:c r="D310" s="97" t="str">
-        <x:v>ABT 1902; Montana</x:v>
-      </x:c>
-      <x:c r="E310" s="97" t="str"/>
+        <x:v>19 JUL 1901; Great Falls, Cascade, Montana</x:v>
+      </x:c>
+      <x:c r="E310" s="97" t="str">
+        <x:v>26 OCT 1991; Washington</x:v>
+      </x:c>
       <x:c r="F310" s="97" t="str">
         <x:v>OWNER-WILLIAM-J-THOREN</x:v>
       </x:c>
       <x:c r="G310" s="97" t="str">
-        <x:v>S28;S32;S33</x:v>
+        <x:v>S28;S32;S33;S34</x:v>
       </x:c>
       <x:c r="H310" s="97" t="str">
-        <x:v>Called Bill in family memory. The 1950 census records him as age 48, born in Montana, and Mary Alice's father.</x:v>
-      </x:c>
-      <x:c r="I310" s="97" t="str"/>
+        <x:v>Called Bill in family memory. The 1910 census places him in Christian and Augusta Thoren's household; later records use William J. or William John.</x:v>
+      </x:c>
+      <x:c r="I310" s="97" t="str">
+        <x:v>F146</x:v>
+      </x:c>
       <x:c r="J310" s="97" t="str">
         <x:v>F145</x:v>
       </x:c>
@@ -35517,27 +35936,509 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="D311" s="97" t="str">
-        <x:v>ABT 1904; Alaska</x:v>
-      </x:c>
-      <x:c r="E311" s="97" t="str"/>
+        <x:v>27 APR 1902; Alaska</x:v>
+      </x:c>
+      <x:c r="E311" s="97" t="str">
+        <x:v>23 AUG 1978; Ocean Park, Pacific, Washington</x:v>
+      </x:c>
       <x:c r="F311" s="97" t="str">
         <x:v>RECORD-ALICE-GALLAHER-THOREN</x:v>
       </x:c>
       <x:c r="G311" s="97" t="str">
-        <x:v>S32;S33</x:v>
+        <x:v>S32;S33;S35</x:v>
       </x:c>
       <x:c r="H311" s="97" t="str">
-        <x:v>The 1950 census records her as age 46, born in Alaska, and Mary Alice's mother; her 1929 marriage record supplies the maiden surname Gallaher.</x:v>
+        <x:v>The 1950 census identifies her as Mary Alice's mother; her 1929 marriage record supplies the maiden surname Gallaher. Her parents remain unproved.</x:v>
       </x:c>
       <x:c r="I311" s="97" t="str"/>
       <x:c r="J311" s="97" t="str">
         <x:v>F145</x:v>
       </x:c>
     </x:row>
+    <x:row r="312">
+      <x:c r="A312" s="97" t="str">
+        <x:v>I338</x:v>
+      </x:c>
+      <x:c r="B312" s="97" t="str">
+        <x:v>Christian Andrew Thoren</x:v>
+      </x:c>
+      <x:c r="C312" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D312" s="97" t="str">
+        <x:v>27 JAN 1861; Ignaberga, Kristianstad, Sweden</x:v>
+      </x:c>
+      <x:c r="E312" s="97" t="str">
+        <x:v>9 MAY 1921; Great Falls, Cascade, Montana</x:v>
+      </x:c>
+      <x:c r="F312" s="97" t="str">
+        <x:v>RECORD-CHRISTIAN-ANDREW-THOREN</x:v>
+      </x:c>
+      <x:c r="G312" s="97" t="str">
+        <x:v>S34;S36</x:v>
+      </x:c>
+      <x:c r="H312" s="97" t="str">
+        <x:v>Swedish records use Christian Andersson and Christian Anders Thorén; U.S. records also use Andrew, Christia, and Christison. | A 1900 census estimate of January 1862 conflicts with the 27 January 1861 indexed Swedish birth and is retained only as a record variation. | The Montana death index misassigns his wife Augusta Nelson as his mother; the Swedish birth record identifies Anders Troedsson and Kjersti Månsdotter as his parents.</x:v>
+      </x:c>
+      <x:c r="I312" s="97" t="str">
+        <x:v>F147</x:v>
+      </x:c>
+      <x:c r="J312" s="97" t="str">
+        <x:v>F146</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313">
+      <x:c r="A313" s="97" t="str">
+        <x:v>I339</x:v>
+      </x:c>
+      <x:c r="B313" s="97" t="str">
+        <x:v>Augusta Nilsdotter</x:v>
+      </x:c>
+      <x:c r="C313" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D313" s="97" t="str">
+        <x:v>30 NOV 1860; Hjärnarp, Kristianstad, Sweden</x:v>
+      </x:c>
+      <x:c r="E313" s="97" t="str">
+        <x:v>4 DEC 1913; Great Falls, Cascade, Montana</x:v>
+      </x:c>
+      <x:c r="F313" s="97" t="str">
+        <x:v>RECORD-AUGUSTA-NILSDOTTER-THOREN</x:v>
+      </x:c>
+      <x:c r="G313" s="97" t="str">
+        <x:v>S34;S37</x:v>
+      </x:c>
+      <x:c r="H313" s="97" t="str">
+        <x:v>The Swedish household record uses the patronymic Nilsdotter; an indexed baptism uses Svensson, and U.S. records use Nilson, Nelson, and Thoren. | A 1900 census estimate of November 1861 conflicts with the 30 November 1860 Swedish birth and baptism records.</x:v>
+      </x:c>
+      <x:c r="I313" s="97" t="str">
+        <x:v>F149</x:v>
+      </x:c>
+      <x:c r="J313" s="97" t="str">
+        <x:v>F146</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="314">
+      <x:c r="A314" s="97" t="str">
+        <x:v>I340</x:v>
+      </x:c>
+      <x:c r="B314" s="97" t="str">
+        <x:v>Anders Troedsson</x:v>
+      </x:c>
+      <x:c r="C314" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D314" s="97" t="str">
+        <x:v>2 MAY 1824; Norra Sandby, Kristianstad, Sweden</x:v>
+      </x:c>
+      <x:c r="E314" s="97" t="str"/>
+      <x:c r="F314" s="97" t="str">
+        <x:v>RECORD-ANDERS-TROEDSSON</x:v>
+      </x:c>
+      <x:c r="G314" s="97" t="str">
+        <x:v>S38</x:v>
+      </x:c>
+      <x:c r="H314" s="97" t="str">
+        <x:v>Household surveys link him first to parents Trued Andersson and Bortha Nilsdotter and later to wife Kjersti Månsdotter and son Christian.</x:v>
+      </x:c>
+      <x:c r="I314" s="97" t="str">
+        <x:v>F148</x:v>
+      </x:c>
+      <x:c r="J314" s="97" t="str">
+        <x:v>F147</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="315">
+      <x:c r="A315" s="97" t="str">
+        <x:v>I341</x:v>
+      </x:c>
+      <x:c r="B315" s="97" t="str">
+        <x:v>Kjersti Månsdotter</x:v>
+      </x:c>
+      <x:c r="C315" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D315" s="97" t="str">
+        <x:v>31 OCT 1825; Mellby, Kristianstad, Sweden</x:v>
+      </x:c>
+      <x:c r="E315" s="97" t="str"/>
+      <x:c r="F315" s="97" t="str">
+        <x:v>RECORD-KJERSTI-MANSDOTTER</x:v>
+      </x:c>
+      <x:c r="G315" s="97" t="str">
+        <x:v>S38</x:v>
+      </x:c>
+      <x:c r="H315" s="97" t="str">
+        <x:v>The reviewed household survey establishes her as Christian's mother; no parent-naming birth or baptism record was located.</x:v>
+      </x:c>
+      <x:c r="I315" s="97" t="str"/>
+      <x:c r="J315" s="97" t="str">
+        <x:v>F147</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="316">
+      <x:c r="A316" s="97" t="str">
+        <x:v>I342</x:v>
+      </x:c>
+      <x:c r="B316" s="97" t="str">
+        <x:v>Trued Andersson</x:v>
+      </x:c>
+      <x:c r="C316" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D316" s="97" t="str">
+        <x:v>25 APR 1792; Norra Sandby, Kristianstad, Sweden</x:v>
+      </x:c>
+      <x:c r="E316" s="97" t="str"/>
+      <x:c r="F316" s="97" t="str">
+        <x:v>RECORD-TRUED-ANDERSSON</x:v>
+      </x:c>
+      <x:c r="G316" s="97" t="str">
+        <x:v>S38</x:v>
+      </x:c>
+      <x:c r="H316" s="97" t="str"/>
+      <x:c r="I316" s="97" t="str"/>
+      <x:c r="J316" s="97" t="str">
+        <x:v>F148</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="317">
+      <x:c r="A317" s="97" t="str">
+        <x:v>I343</x:v>
+      </x:c>
+      <x:c r="B317" s="97" t="str">
+        <x:v>Bortha Nilsdotter</x:v>
+      </x:c>
+      <x:c r="C317" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D317" s="97" t="str">
+        <x:v>1783; Gumlösa, Kristianstad, Sweden</x:v>
+      </x:c>
+      <x:c r="E317" s="97" t="str"/>
+      <x:c r="F317" s="97" t="str">
+        <x:v>RECORD-BORTHA-NILSDOTTER</x:v>
+      </x:c>
+      <x:c r="G317" s="97" t="str">
+        <x:v>S38</x:v>
+      </x:c>
+      <x:c r="H317" s="97" t="str">
+        <x:v>No parent-naming baptism record was located; same-name baptism hints from other parishes were rejected.</x:v>
+      </x:c>
+      <x:c r="I317" s="97" t="str"/>
+      <x:c r="J317" s="97" t="str">
+        <x:v>F148</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="318">
+      <x:c r="A318" s="97" t="str">
+        <x:v>I344</x:v>
+      </x:c>
+      <x:c r="B318" s="97" t="str">
+        <x:v>Nils Svensson</x:v>
+      </x:c>
+      <x:c r="C318" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D318" s="97" t="str">
+        <x:v>3 MAY 1825; Ränneslöv, Halland, Sweden</x:v>
+      </x:c>
+      <x:c r="E318" s="97" t="str"/>
+      <x:c r="F318" s="97" t="str">
+        <x:v>RECORD-NILS-SVENSSON</x:v>
+      </x:c>
+      <x:c r="G318" s="97" t="str">
+        <x:v>S39;S40</x:v>
+      </x:c>
+      <x:c r="H318" s="97" t="str">
+        <x:v>His baptism names Gunnilla Nilsdotter as mother but does not name a father; the unknown father remains blank despite the patronymic Svensson.</x:v>
+      </x:c>
+      <x:c r="I318" s="97" t="str">
+        <x:v>F150</x:v>
+      </x:c>
+      <x:c r="J318" s="97" t="str">
+        <x:v>F149</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="319">
+      <x:c r="A319" s="97" t="str">
+        <x:v>I345</x:v>
+      </x:c>
+      <x:c r="B319" s="97" t="str">
+        <x:v>Christina Persdotter</x:v>
+      </x:c>
+      <x:c r="C319" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D319" s="97" t="str">
+        <x:v>24 JAN 1823; Hasslöv, Halland, Sweden</x:v>
+      </x:c>
+      <x:c r="E319" s="97" t="str"/>
+      <x:c r="F319" s="97" t="str">
+        <x:v>RECORD-CHRISTINA-PERSDOTTER</x:v>
+      </x:c>
+      <x:c r="G319" s="97" t="str">
+        <x:v>S39;S42</x:v>
+      </x:c>
+      <x:c r="H319" s="97" t="str">
+        <x:v>Indexed records also use Kristina Persdotter and Stina Parsdotter.</x:v>
+      </x:c>
+      <x:c r="I319" s="97" t="str">
+        <x:v>F152</x:v>
+      </x:c>
+      <x:c r="J319" s="97" t="str">
+        <x:v>F149</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="320">
+      <x:c r="A320" s="97" t="str">
+        <x:v>I346</x:v>
+      </x:c>
+      <x:c r="B320" s="97" t="str">
+        <x:v>Gunnilla Nilsdotter</x:v>
+      </x:c>
+      <x:c r="C320" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D320" s="97" t="str">
+        <x:v>20 SEP 1796; Ränneslöv, Halland, Sweden</x:v>
+      </x:c>
+      <x:c r="E320" s="97" t="str"/>
+      <x:c r="F320" s="97" t="str">
+        <x:v>RECORD-GUNNILLA-NILSDOTTER</x:v>
+      </x:c>
+      <x:c r="G320" s="97" t="str">
+        <x:v>S40;S41</x:v>
+      </x:c>
+      <x:c r="H320" s="97" t="str">
+        <x:v>Indexed records also use Gunla Nilsdotter. She is the only parent named in Nils Svensson's baptism.</x:v>
+      </x:c>
+      <x:c r="I320" s="97" t="str">
+        <x:v>F151</x:v>
+      </x:c>
+      <x:c r="J320" s="97" t="str">
+        <x:v>F150</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="321">
+      <x:c r="A321" s="97" t="str">
+        <x:v>I347</x:v>
+      </x:c>
+      <x:c r="B321" s="97" t="str">
+        <x:v>Nils Johansson</x:v>
+      </x:c>
+      <x:c r="C321" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D321" s="97" t="str"/>
+      <x:c r="E321" s="97" t="str"/>
+      <x:c r="F321" s="97" t="str">
+        <x:v>RECORD-NILS-JOHANSSON</x:v>
+      </x:c>
+      <x:c r="G321" s="97" t="str">
+        <x:v>S41</x:v>
+      </x:c>
+      <x:c r="H321" s="97" t="str">
+        <x:v>Named as Gunnilla Nilsdotter's father in her 1796 baptism; no further identity was proved.</x:v>
+      </x:c>
+      <x:c r="I321" s="97" t="str"/>
+      <x:c r="J321" s="97" t="str">
+        <x:v>F151</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="322">
+      <x:c r="A322" s="97" t="str">
+        <x:v>I348</x:v>
+      </x:c>
+      <x:c r="B322" s="97" t="str">
+        <x:v>Elna Nilsdotter</x:v>
+      </x:c>
+      <x:c r="C322" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D322" s="97" t="str"/>
+      <x:c r="E322" s="97" t="str"/>
+      <x:c r="F322" s="97" t="str">
+        <x:v>RECORD-ELNA-NILSDOTTER</x:v>
+      </x:c>
+      <x:c r="G322" s="97" t="str">
+        <x:v>S41</x:v>
+      </x:c>
+      <x:c r="H322" s="97" t="str">
+        <x:v>Named as Gunnilla Nilsdotter's mother in her 1796 baptism; no further identity was proved.</x:v>
+      </x:c>
+      <x:c r="I322" s="97" t="str"/>
+      <x:c r="J322" s="97" t="str">
+        <x:v>F151</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323">
+      <x:c r="A323" s="97" t="str">
+        <x:v>I349</x:v>
+      </x:c>
+      <x:c r="B323" s="97" t="str">
+        <x:v>Pehr Erlandsson</x:v>
+      </x:c>
+      <x:c r="C323" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D323" s="97" t="str">
+        <x:v>10 FEB 1790; Hishult, Halland, Sweden</x:v>
+      </x:c>
+      <x:c r="E323" s="97" t="str"/>
+      <x:c r="F323" s="97" t="str">
+        <x:v>RECORD-PEHR-ERLANDSSON</x:v>
+      </x:c>
+      <x:c r="G323" s="97" t="str">
+        <x:v>S43;S44</x:v>
+      </x:c>
+      <x:c r="H323" s="97" t="str">
+        <x:v>A household survey reports 10 February 1791; the 1790 baptism is nearer to the event and controls the canonical birth date.</x:v>
+      </x:c>
+      <x:c r="I323" s="97" t="str">
+        <x:v>F153</x:v>
+      </x:c>
+      <x:c r="J323" s="97" t="str">
+        <x:v>F152</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="324">
+      <x:c r="A324" s="97" t="str">
+        <x:v>I350</x:v>
+      </x:c>
+      <x:c r="B324" s="97" t="str">
+        <x:v>Ingier Hansdotter</x:v>
+      </x:c>
+      <x:c r="C324" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D324" s="97" t="str">
+        <x:v>20 MAR 1794; Hasslöv, Halland, Sweden</x:v>
+      </x:c>
+      <x:c r="E324" s="97" t="str"/>
+      <x:c r="F324" s="97" t="str">
+        <x:v>RECORD-INGIER-HANSDOTTER</x:v>
+      </x:c>
+      <x:c r="G324" s="97" t="str">
+        <x:v>S43;S45</x:v>
+      </x:c>
+      <x:c r="H324" s="97" t="str"/>
+      <x:c r="I324" s="97" t="str">
+        <x:v>F154</x:v>
+      </x:c>
+      <x:c r="J324" s="97" t="str">
+        <x:v>F152</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="325">
+      <x:c r="A325" s="97" t="str">
+        <x:v>I351</x:v>
+      </x:c>
+      <x:c r="B325" s="97" t="str">
+        <x:v>Erland Pålsson</x:v>
+      </x:c>
+      <x:c r="C325" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D325" s="97" t="str"/>
+      <x:c r="E325" s="97" t="str"/>
+      <x:c r="F325" s="97" t="str">
+        <x:v>RECORD-ERLAND-PALSSON</x:v>
+      </x:c>
+      <x:c r="G325" s="97" t="str">
+        <x:v>S44</x:v>
+      </x:c>
+      <x:c r="H325" s="97" t="str">
+        <x:v>Named as Pehr Erlandsson's father in the 1790 baptism. A possible 1756 Knäred baptism was not linked closely enough to import its parents.</x:v>
+      </x:c>
+      <x:c r="I325" s="97" t="str"/>
+      <x:c r="J325" s="97" t="str">
+        <x:v>F153</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326">
+      <x:c r="A326" s="97" t="str">
+        <x:v>I352</x:v>
+      </x:c>
+      <x:c r="B326" s="97" t="str">
+        <x:v>Bengta Pehrsdotter</x:v>
+      </x:c>
+      <x:c r="C326" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D326" s="97" t="str"/>
+      <x:c r="E326" s="97" t="str"/>
+      <x:c r="F326" s="97" t="str">
+        <x:v>RECORD-BENGTA-PEHRSDOTTER</x:v>
+      </x:c>
+      <x:c r="G326" s="97" t="str">
+        <x:v>S44</x:v>
+      </x:c>
+      <x:c r="H326" s="97" t="str">
+        <x:v>Named as Pehr Erlandsson's mother in the 1790 baptism. A similar Bengta Persdotter baptism and marriage belonged to another woman and was rejected.</x:v>
+      </x:c>
+      <x:c r="I326" s="97" t="str"/>
+      <x:c r="J326" s="97" t="str">
+        <x:v>F153</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327">
+      <x:c r="A327" s="97" t="str">
+        <x:v>I353</x:v>
+      </x:c>
+      <x:c r="B327" s="97" t="str">
+        <x:v>Hans Månsson</x:v>
+      </x:c>
+      <x:c r="C327" s="97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D327" s="97" t="str"/>
+      <x:c r="E327" s="97" t="str"/>
+      <x:c r="F327" s="97" t="str">
+        <x:v>RECORD-HANS-MANSSON</x:v>
+      </x:c>
+      <x:c r="G327" s="97" t="str">
+        <x:v>S45</x:v>
+      </x:c>
+      <x:c r="H327" s="97" t="str">
+        <x:v>Named as Ingier Hansdotter's father in her 1794 baptism; no further identity was proved.</x:v>
+      </x:c>
+      <x:c r="I327" s="97" t="str"/>
+      <x:c r="J327" s="97" t="str">
+        <x:v>F154</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328">
+      <x:c r="A328" s="97" t="str">
+        <x:v>I354</x:v>
+      </x:c>
+      <x:c r="B328" s="97" t="str">
+        <x:v>Maria Hansdotter</x:v>
+      </x:c>
+      <x:c r="C328" s="97" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D328" s="97" t="str"/>
+      <x:c r="E328" s="97" t="str"/>
+      <x:c r="F328" s="97" t="str">
+        <x:v>RECORD-MARIA-HANSDOTTER</x:v>
+      </x:c>
+      <x:c r="G328" s="97" t="str">
+        <x:v>S45</x:v>
+      </x:c>
+      <x:c r="H328" s="97" t="str">
+        <x:v>Named as Ingier Hansdotter's mother in her 1794 baptism; no further identity was proved.</x:v>
+      </x:c>
+      <x:c r="I328" s="97" t="str"/>
+      <x:c r="J328" s="97" t="str">
+        <x:v>F154</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b7c03ac683240ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R501339a4b9cf45c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>